<commit_message>
Update current cap sources and reconcile October 10 coherence review
</commit_message>
<xml_diff>
--- a/project_current/coherence/Coherence_Tracker.xlsx
+++ b/project_current/coherence/Coherence_Tracker.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coherence items" sheetId="1" r:id="Rd227d21a59fa48a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coherence items" sheetId="1" r:id="R20c869f04f9a4fd0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -201,7 +201,7 @@
         <x:color rgb="FF8B3D16"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE7D9"/>
         </x:patternFill>
       </x:fill>
@@ -211,7 +211,7 @@
         <x:color rgb="FF57466C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFECE8F4"/>
         </x:patternFill>
       </x:fill>
@@ -221,7 +221,7 @@
         <x:color rgb="FF4B5A67"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE9EEF2"/>
         </x:patternFill>
       </x:fill>
@@ -232,7 +232,7 @@
         <x:color rgb="FF9B2226"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFBE3E3"/>
         </x:patternFill>
       </x:fill>
@@ -243,7 +243,7 @@
         <x:color rgb="FF9B2226"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFBE3E3"/>
         </x:patternFill>
       </x:fill>
@@ -517,7 +517,7 @@
     </x:row>
     <x:row r="3" ht="18.75" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>Baseline review: 9 October 2026. Current items and recorded decisions are kept here.</x:v>
+        <x:v>Review updated: 10 October 2026. Source selections, recorded responses and closure evidence are preserved here.</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -537,7 +537,7 @@
       </x:c>
       <x:c r="B4" s="31" t="n">
         <x:f>COUNTIFS($A$9:$A$1008,"&lt;&gt;",$B$9:$B$1008,"&lt;&gt;Closed",$B$9:$B$1008,"&lt;&gt;Not applicable")</x:f>
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C4" s="2" t="str">
         <x:v>Awaiting source</x:v>
@@ -551,14 +551,14 @@
       </x:c>
       <x:c r="F4" s="31" t="n">
         <x:f>COUNTIFS($A$9:$A$1008,"&lt;&gt;",$B$9:$B$1008,"Deferred")</x:f>
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G4" s="2" t="str">
         <x:v>Marked closed / N.A.</x:v>
       </x:c>
       <x:c r="H4" s="31" t="n">
         <x:f>COUNTIFS($A$9:$A$1008,"&lt;&gt;",$B$9:$B$1008,"Closed")+COUNTIFS($A$9:$A$1008,"&lt;&gt;",$B$9:$B$1008,"Not applicable")</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I4" s="2"/>
       <x:c r="J4" s="2"/>
@@ -649,12 +649,12 @@
         <x:v>Last reviewed</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="67.5" customHeight="1">
+    <x:row r="9" ht="116" customHeight="1">
       <x:c r="A9" s="18" t="str">
         <x:v>COH-001</x:v>
       </x:c>
       <x:c r="B9" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Closed</x:v>
       </x:c>
       <x:c r="C9" s="19" t="str">
         <x:v>Pier</x:v>
@@ -663,23 +663,27 @@
         <x:v>Right bearing-row offset</x:v>
       </x:c>
       <x:c r="E9" s="19" t="str">
-        <x:v>Model right row is +10.14 in; journal is +10.50 in. Difference is 0.36 in. Left row agrees at -10.50 in.</x:v>
+        <x:v>Historical right row was +10.14 in. The matching Pier_Fixed.XML now has nodes 183/184 at +10.50 in and nodes 181/182 at -10.50 in, matching the journal.</x:v>
       </x:c>
       <x:c r="F9" s="19" t="str">
-        <x:v>Choose the intended offset, then reconcile the model/journal and affected load transfers.</x:v>
-      </x:c>
-      <x:c r="G9" s="27"/>
+        <x:v>Coordinate discrepancy resolved. Full model load and convergence review remains COH-004.</x:v>
+      </x:c>
+      <x:c r="G9" s="27" t="str">
+        <x:v>I need to correct the FBMP model I think there is a typo in it. I'll update the model and reupload the report. — recorded response, 9 October 2026.</x:v>
+      </x:c>
       <x:c r="H9" s="27"/>
       <x:c r="I9" s="28"/>
-      <x:c r="J9" s="27"/>
+      <x:c r="J9" s="27" t="str">
+        <x:v>10 October: exact report/XML fingerprint matched; PIER-XML nodal coordinates 181–184 verified. See source_update.json.</x:v>
+      </x:c>
       <x:c r="K9" s="19" t="str">
-        <x:v>PIER-XML; JOURNAL; coherence/evidence/pier_review_2026-10-09.xlsx, item 02</x:v>
+        <x:v>PIER-XML; JOURNAL; coherence/evidence/pier_review_2026-10-09.xlsx, item 02; tasks/T006/response-disposition.json, item 02; coherence/evidence/2026-10-10/source_update.json</x:v>
       </x:c>
       <x:c r="L9" s="28" t="n">
-        <x:v>46304.5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="67.5" customHeight="1">
+        <x:v>46305</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="116" customHeight="1">
       <x:c r="A10" s="24" t="str">
         <x:v>COH-002</x:v>
       </x:c>
@@ -693,23 +697,25 @@
         <x:v>U-bar / pile conflicts</x:v>
       </x:c>
       <x:c r="E10" s="25" t="str">
-        <x:v>Report R2/R4/R6/R8 U-bars intersect pile-clearance envelopes. End-bent hook direction has not been applied to the pier.</x:v>
+        <x:v>The new pier cage uses #5 U-bars with 50-degree trial hook rotations. Hook development and engagement remain pending. Field bending was permitted in the recorded T006 response.</x:v>
       </x:c>
       <x:c r="F10" s="25" t="str">
-        <x:v>Provide or develop the pier hook detail and check clearance, development and anchorage.</x:v>
-      </x:c>
-      <x:c r="G10" s="27"/>
+        <x:v>Verify the revised U-bar clearance, development and engagement. Separate end-face U-grid failure is COH-019.</x:v>
+      </x:c>
+      <x:c r="G10" s="27" t="str">
+        <x:v>U bars tails can be field bent to accommodate a potential clash — recorded response, 9 October 2026.</x:v>
+      </x:c>
       <x:c r="H10" s="27"/>
       <x:c r="I10" s="28"/>
       <x:c r="J10" s="27"/>
       <x:c r="K10" s="25" t="str">
-        <x:v>PIER-REPORT; coherence/evidence/pier_review_2026-10-09.xlsx, item 03</x:v>
+        <x:v>PIER-REPORT; coherence/evidence/pier_review_2026-10-09.xlsx, item 03; tasks/T006/response-disposition.json, item 03; coherence/evidence/2026-10-10/source_update.json</x:v>
       </x:c>
       <x:c r="L10" s="28" t="n">
-        <x:v>46304.5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="67.5" customHeight="1">
+        <x:v>46305</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="116" customHeight="1">
       <x:c r="A11" s="18" t="str">
         <x:v>COH-003</x:v>
       </x:c>
@@ -723,23 +729,25 @@
         <x:v>Longitudinal tension reference</x:v>
       </x:c>
       <x:c r="E11" s="19" t="str">
-        <x:v>Historical report reference: required 4.287 in2; credited 3.080 in2; shortfall 1.207 in2. This is a reference check, not an established actual-cage failure.</x:v>
+        <x:v>Historical uniform-reference shortfall is retained in prior evidence. New actual-cage longitudinal tension is PENDING: N 0.946947, P 0.776624, B 0.863733. Ratios below 1 do not close prerequisites.</x:v>
       </x:c>
       <x:c r="F11" s="19" t="str">
-        <x:v>Evaluate the actual cage/load path or document the disposition of the reference check.</x:v>
-      </x:c>
-      <x:c r="G11" s="27"/>
+        <x:v>Resolve developed-steel and load-path prerequisites and document actual-cage acceptance.</x:v>
+      </x:c>
+      <x:c r="G11" s="27" t="str">
+        <x:v>Explain to me in chat what the N uniform check is all about — recorded response, 9 October 2026.</x:v>
+      </x:c>
       <x:c r="H11" s="27"/>
       <x:c r="I11" s="28"/>
       <x:c r="J11" s="27"/>
       <x:c r="K11" s="19" t="str">
-        <x:v>PIER-REPORT; coherence/evidence/pier_review_2026-10-09.xlsx, item 04</x:v>
+        <x:v>PIER-REPORT; coherence/evidence/pier_review_2026-10-09.xlsx, item 04; tasks/T006/response-disposition.json, item 04; coherence/evidence/2026-10-10/source_update.json</x:v>
       </x:c>
       <x:c r="L11" s="28" t="n">
-        <x:v>46304.5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="67.5" customHeight="1">
+        <x:v>46305</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="116" customHeight="1">
       <x:c r="A12" s="24" t="str">
         <x:v>COH-004</x:v>
       </x:c>
@@ -753,23 +761,25 @@
         <x:v>Complete model load comparison</x:v>
       </x:c>
       <x:c r="E12" s="25" t="str">
-        <x:v>Exact XML identity is established. Full wind, below-pad weights, transfer moments, combinations and convergence remain unverified against the current journal.</x:v>
+        <x:v>New Pier_Fixed report/XML fingerprints match and bearing offsets reconcile. Full current wind, below-pad weights, transfer moments, combinations and convergence remain unverified against T006.</x:v>
       </x:c>
       <x:c r="F12" s="25" t="str">
-        <x:v>Compare the adopted load inputs and document any corrections and required rerun.</x:v>
-      </x:c>
-      <x:c r="G12" s="27"/>
+        <x:v>Compare the exact current model loading with T006 and document needed reruns and convergence evidence.</x:v>
+      </x:c>
+      <x:c r="G12" s="27" t="str">
+        <x:v>Will need to provide an update cap design report as the latest. — recorded response, 9 October 2026.</x:v>
+      </x:c>
       <x:c r="H12" s="27"/>
       <x:c r="I12" s="28"/>
       <x:c r="J12" s="27"/>
       <x:c r="K12" s="25" t="str">
-        <x:v>PIER-XML; JOURNAL; coherence/evidence/pier_review_2026-10-09.xlsx, item 05</x:v>
+        <x:v>PIER-XML; JOURNAL; coherence/evidence/pier_review_2026-10-09.xlsx, item 05; tasks/T006/response-disposition.json, item 05; coherence/evidence/2026-10-10/source_update.json</x:v>
       </x:c>
       <x:c r="L12" s="28" t="n">
-        <x:v>46304.5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="67.5" customHeight="1">
+        <x:v>46305</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="116" customHeight="1">
       <x:c r="A13" s="18" t="str">
         <x:v>COH-005</x:v>
       </x:c>
@@ -783,28 +793,32 @@
         <x:v>Wind and wall geometry</x:v>
       </x:c>
       <x:c r="E13" s="19" t="str">
-        <x:v>Cap length is 230 in; retained wind face is 231 in. Wall, fin and crash-wall dimensions may represent different envelopes.</x:v>
+        <x:v>T006 linked wind width to the 230-in cap length. The 231-in discrepancy is resolved in the accepted journal. Separate wall/fin dimensions and model wind-load currency remain open.</x:v>
       </x:c>
       <x:c r="F13" s="19" t="str">
-        <x:v>Establish the wall/wind dimensions and update only the affected loads and quantities.</x:v>
-      </x:c>
-      <x:c r="G13" s="27"/>
+        <x:v>Establish remaining wall/fin geometry and compare current model wind loads with the T006 basis.</x:v>
+      </x:c>
+      <x:c r="G13" s="27" t="str">
+        <x:v>Use the cap length from the report — recorded response, 9 October 2026.</x:v>
+      </x:c>
       <x:c r="H13" s="27"/>
       <x:c r="I13" s="28"/>
-      <x:c r="J13" s="27"/>
+      <x:c r="J13" s="27" t="str">
+        <x:v>Partial: T006 receipt and final review verify 230-in width and dependent wind quantities; wall quantities were excluded.</x:v>
+      </x:c>
       <x:c r="K13" s="19" t="str">
-        <x:v>JOURNAL; coherence/evidence/pier_review_2026-10-09.xlsx, item 06</x:v>
+        <x:v>JOURNAL; coherence/evidence/pier_review_2026-10-09.xlsx, item 06; tasks/T006/response-disposition.json, item 06; coherence/evidence/2026-10-10/source_update.json</x:v>
       </x:c>
       <x:c r="L13" s="28" t="n">
-        <x:v>46304.5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="67.5" customHeight="1">
+        <x:v>46305</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="116" customHeight="1">
       <x:c r="A14" s="24" t="str">
         <x:v>COH-006</x:v>
       </x:c>
       <x:c r="B14" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Closed</x:v>
       </x:c>
       <x:c r="C14" s="25" t="str">
         <x:v>Journal</x:v>
@@ -813,28 +827,32 @@
         <x:v>Historical quantity sketches</x:v>
       </x:c>
       <x:c r="E14" s="25" t="str">
-        <x:v>The quantity sheet retains earlier three-beam / 19-ft-3-in sketches. Live cap quantity is 230 ft3.</x:v>
+        <x:v>T006 labeled the older cap sketches historical; the live cap quantity remains 230 ft3.</x:v>
       </x:c>
       <x:c r="F14" s="25" t="str">
-        <x:v>Update or explicitly label the historical sketches without changing current calculation records.</x:v>
-      </x:c>
-      <x:c r="G14" s="27"/>
+        <x:v>No action for historical labels. Separate wall quantities remain open.</x:v>
+      </x:c>
+      <x:c r="G14" s="27" t="str">
+        <x:v>Use the cap length from the report — recorded response, 9 October 2026.</x:v>
+      </x:c>
       <x:c r="H14" s="27"/>
       <x:c r="I14" s="28"/>
-      <x:c r="J14" s="27"/>
+      <x:c r="J14" s="27" t="str">
+        <x:v>Existing T006 acceptance fingerprint and all listed evidence hashes verified. Accepted final review records native inspection of the quantity note.</x:v>
+      </x:c>
       <x:c r="K14" s="25" t="str">
-        <x:v>JOURNAL; coherence/evidence/pier_review_2026-10-09.xlsx, item 06</x:v>
+        <x:v>JOURNAL; coherence/evidence/pier_review_2026-10-09.xlsx, item 06; tasks/T006/response-disposition.json, item 06; coherence/evidence/2026-10-10/source_update.json</x:v>
       </x:c>
       <x:c r="L14" s="28" t="n">
-        <x:v>46304.5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="67.5" customHeight="1">
+        <x:v>46305</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="116" customHeight="1">
       <x:c r="A15" s="18" t="str">
         <x:v>COH-007</x:v>
       </x:c>
       <x:c r="B15" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Deferred</x:v>
       </x:c>
       <x:c r="C15" s="19" t="str">
         <x:v>Pier</x:v>
@@ -843,28 +861,30 @@
         <x:v>Remaining design checks</x:v>
       </x:c>
       <x:c r="E15" s="19" t="str">
-        <x:v>Historical report has 48 pending/conditional checks. Service III is already N/A by recorded direction. Other detail, fatigue, load-path and omitted-action checks remain open.</x:v>
+        <x:v>New pier report: 67 pending entries and two FAIL entries (one end-grid clearance failure and its aggregate summary). Service III remains N/A by D-007 despite the report label.</x:v>
       </x:c>
       <x:c r="F15" s="19" t="str">
-        <x:v>Separate the remaining checks into actionable items and document applicable criteria and completion evidence.</x:v>
-      </x:c>
-      <x:c r="G15" s="27"/>
+        <x:v>Retain the recorded deferral. Resolve individual checks when directed; address new end-grid failure under COH-019.</x:v>
+      </x:c>
+      <x:c r="G15" s="27" t="str">
+        <x:v>Leave as is — recorded response, 9 October 2026.</x:v>
+      </x:c>
       <x:c r="H15" s="27"/>
       <x:c r="I15" s="28"/>
       <x:c r="J15" s="27"/>
       <x:c r="K15" s="19" t="str">
-        <x:v>PIER-REPORT; coherence/evidence/pier_review_2026-10-09.xlsx, item 07</x:v>
+        <x:v>PIER-REPORT; coherence/evidence/pier_review_2026-10-09.xlsx, item 07; tasks/T006/response-disposition.json, item 07; coherence/evidence/2026-10-10/source_update.json</x:v>
       </x:c>
       <x:c r="L15" s="28" t="n">
-        <x:v>46304.5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="67.5" customHeight="1">
+        <x:v>46305</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="116" customHeight="1">
       <x:c r="A16" s="24" t="str">
         <x:v>COH-008</x:v>
       </x:c>
       <x:c r="B16" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Deferred</x:v>
       </x:c>
       <x:c r="C16" s="25" t="str">
         <x:v>Pier</x:v>
@@ -873,28 +893,30 @@
         <x:v>Spacing and fabrication takeoff</x:v>
       </x:c>
       <x:c r="E16" s="25" t="str">
-        <x:v>Adjacent-run clearance is 2.00 in, equal to the entered minimum. The gross 1171.89-lb steel estimate omits laps, closures, undrawn anchorage and waste.</x:v>
+        <x:v>New pier gross steel is 1260.94 lb and excludes laps, closures, undrawn anchorage and waste. Spacing/fabrication review remains deferred to shops by recorded direction.</x:v>
       </x:c>
       <x:c r="F16" s="25" t="str">
-        <x:v>Confirm tolerance/spacing allowance and complete the fabrication takeoff if required.</x:v>
-      </x:c>
-      <x:c r="G16" s="27"/>
+        <x:v>Complete the tolerance and fabrication takeoff review at shops, preserving the deferral.</x:v>
+      </x:c>
+      <x:c r="G16" s="27" t="str">
+        <x:v>Leave as is we can deal with this issue in shops later — recorded response, 9 October 2026.</x:v>
+      </x:c>
       <x:c r="H16" s="27"/>
       <x:c r="I16" s="28"/>
       <x:c r="J16" s="27"/>
       <x:c r="K16" s="25" t="str">
-        <x:v>PIER-REPORT; coherence/evidence/pier_review_2026-10-09.xlsx, item 08</x:v>
+        <x:v>PIER-REPORT; coherence/evidence/pier_review_2026-10-09.xlsx, item 08; tasks/T006/response-disposition.json, item 08; coherence/evidence/2026-10-10/source_update.json</x:v>
       </x:c>
       <x:c r="L16" s="28" t="n">
-        <x:v>46304.5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="67.5" customHeight="1">
+        <x:v>46305</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="116" customHeight="1">
       <x:c r="A17" s="18" t="str">
         <x:v>COH-009</x:v>
       </x:c>
       <x:c r="B17" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Closed</x:v>
       </x:c>
       <x:c r="C17" s="19" t="str">
         <x:v>Journal</x:v>
@@ -903,20 +925,24 @@
         <x:v>Three reference links</x:v>
       </x:c>
       <x:c r="E17" s="19" t="str">
-        <x:v>Three inherited LoadCombinations links remain unresolved: CodePage42 twice and CodePage14 once. The prior 110 stored errors were removed with retired modules.</x:v>
+        <x:v>T006 repaired the two CodePage42 references and the CodePage14 reference using verified existing targets.</x:v>
       </x:c>
       <x:c r="F17" s="19" t="str">
-        <x:v>Identify and repair the intended references through the existing journal workflow.</x:v>
-      </x:c>
-      <x:c r="G17" s="27"/>
+        <x:v>No action for these three historical links.</x:v>
+      </x:c>
+      <x:c r="G17" s="27" t="str">
+        <x:v>repair now — recorded response, 9 October 2026.</x:v>
+      </x:c>
       <x:c r="H17" s="27"/>
       <x:c r="I17" s="28"/>
-      <x:c r="J17" s="27"/>
+      <x:c r="J17" s="27" t="str">
+        <x:v>Existing T006 acceptance and evidence hashes verified; its final review records zero stored errors and zero broken links.</x:v>
+      </x:c>
       <x:c r="K17" s="19" t="str">
-        <x:v>JOURNAL; coherence/evidence/pier_review_2026-10-09.xlsx, item 09; coherence/evidence/end_bent_response_review.md</x:v>
+        <x:v>JOURNAL; coherence/evidence/pier_review_2026-10-09.xlsx, item 09; coherence/evidence/end_bent_response_review.md; tasks/T006/response-disposition.json, item 09; coherence/evidence/2026-10-10/source_update.json</x:v>
       </x:c>
       <x:c r="L17" s="28" t="n">
-        <x:v>46304.5</x:v>
+        <x:v>46305</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="67.5" customHeight="1">
@@ -948,10 +974,10 @@
         <x:v>JOURNAL; coherence/evidence/end_bent_response_review.md, item 02</x:v>
       </x:c>
       <x:c r="L18" s="28" t="n">
-        <x:v>46304.5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="67.5" customHeight="1">
+        <x:v>46304</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="116" customHeight="1">
       <x:c r="A19" s="18" t="str">
         <x:v>COH-011</x:v>
       </x:c>
@@ -965,10 +991,10 @@
         <x:v>Revised U-bar hooks</x:v>
       </x:c>
       <x:c r="E19" s="19" t="str">
-        <x:v>Field adjustment of interfering hooks is the recorded direction. Revised coordinates, clearance and anchorage verification have not been supplied.</x:v>
+        <x:v>The new end-bent report includes #5 U-bars with 50-degree trial rotations and 3.75-in tails. Rotated-hook development and engagement remain PENDING.</x:v>
       </x:c>
       <x:c r="F19" s="19" t="str">
-        <x:v>Document the adjusted detail and verify clearance/development/anchorage.</x:v>
+        <x:v>Verify revised hook clearance, development and engagement. Separate end-face U-grid failure is COH-020.</x:v>
       </x:c>
       <x:c r="G19" s="27" t="str">
         <x:v>Field-bend interfering hooks for clearance — recorded user direction, 8 October 2026.</x:v>
@@ -977,13 +1003,13 @@
       <x:c r="I19" s="28"/>
       <x:c r="J19" s="27"/>
       <x:c r="K19" s="19" t="str">
-        <x:v>EB-REPORT; coherence/evidence/end_bent_response_review.md, item 06</x:v>
+        <x:v>EB-REPORT; coherence/evidence/end_bent_response_review.md, item 06; coherence/evidence/2026-10-10/source_update.json</x:v>
       </x:c>
       <x:c r="L19" s="28" t="n">
-        <x:v>46304.5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="67.5" customHeight="1">
+        <x:v>46305</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="116" customHeight="1">
       <x:c r="A20" s="24" t="str">
         <x:v>COH-012</x:v>
       </x:c>
@@ -997,23 +1023,23 @@
         <x:v>Remaining design checks</x:v>
       </x:c>
       <x:c r="E20" s="25" t="str">
-        <x:v>Service III is already N/A. Fatigue, anchorage/development, D-regions, force zones, exposure/code basis and omitted-action checks remain separate.</x:v>
+        <x:v>New end-bent report: 50 pending entries and two FAIL entries (end-grid clearance and aggregate summary). Service III remains N/A by D-007; other pending checks remain separate.</x:v>
       </x:c>
       <x:c r="F20" s="25" t="str">
-        <x:v>Record a disposition and evidence for each applicable outstanding design check.</x:v>
+        <x:v>Record evidence/disposition for remaining fatigue, anchorage, shear prerequisites, face reinforcement, D-regions and exposure checks.</x:v>
       </x:c>
       <x:c r="G20" s="27"/>
       <x:c r="H20" s="27"/>
       <x:c r="I20" s="28"/>
       <x:c r="J20" s="27"/>
       <x:c r="K20" s="25" t="str">
-        <x:v>EB-REPORT; coherence/evidence/end_bent_response_review.md, item 07</x:v>
+        <x:v>EB-REPORT; coherence/evidence/end_bent_response_review.md, item 07; coherence/evidence/2026-10-10/source_update.json</x:v>
       </x:c>
       <x:c r="L20" s="28" t="n">
-        <x:v>46304.5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="67.5" customHeight="1">
+        <x:v>46305</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="116" customHeight="1">
       <x:c r="A21" s="18" t="str">
         <x:v>COH-013</x:v>
       </x:c>
@@ -1027,23 +1053,23 @@
         <x:v>Matching raw analysis export</x:v>
       </x:c>
       <x:c r="E21" s="19" t="str">
-        <x:v>The report is adopted as the current source, but its exact analyzed XML is absent. The available same-named file has a different fingerprint.</x:v>
+        <x:v>New end-bent report requires XML SHA256 8414fbedfbf1270fbd65b2cf940f2dc2050818c282cc6f66db2d20b2f3ff17ee. Available same-named XML matches only the superseded report.</x:v>
       </x:c>
       <x:c r="F21" s="19" t="str">
-        <x:v>Add the exact matching XML and its native input/run record. Expected hash is in source_register.csv.</x:v>
+        <x:v>Supply the matching new End Bent 1 XML and native run record; do not substitute the older export.</x:v>
       </x:c>
       <x:c r="G21" s="27"/>
       <x:c r="H21" s="27"/>
       <x:c r="I21" s="28"/>
       <x:c r="J21" s="27"/>
       <x:c r="K21" s="19" t="str">
-        <x:v>EB-REPORT; EB-XML; coherence/evidence/end_bent_provenance.json</x:v>
+        <x:v>EB-REPORT; EB-XML; coherence/evidence/end_bent_provenance.json; coherence/evidence/2026-10-10/source_update.json</x:v>
       </x:c>
       <x:c r="L21" s="28" t="n">
-        <x:v>46304.5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="67.5" customHeight="1">
+        <x:v>46305</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="116" customHeight="1">
       <x:c r="A22" s="24" t="str">
         <x:v>COH-014</x:v>
       </x:c>
@@ -1057,10 +1083,10 @@
         <x:v>Common controlling design basis</x:v>
       </x:c>
       <x:c r="E22" s="25" t="str">
-        <x:v>The user adopted the controlling End Bent 1 configuration for both ends. Independent End Bent 2 action verification remains outside the recorded review.</x:v>
+        <x:v>D-004 common end-bent design direction is preserved. New End Bent 1 data do not establish that its actions bound End Bent 2.</x:v>
       </x:c>
       <x:c r="F22" s="25" t="str">
-        <x:v>Document how End Bent 1 bounds the relevant End Bent 2 actions and conditions.</x:v>
+        <x:v>Document how the revised End Bent 1 actions bound both end bents.</x:v>
       </x:c>
       <x:c r="G22" s="27" t="str">
         <x:v>Use the common controlling end-bent design — recorded user direction, 8 October 2026.</x:v>
@@ -1069,10 +1095,10 @@
       <x:c r="I22" s="28"/>
       <x:c r="J22" s="27"/>
       <x:c r="K22" s="25" t="str">
-        <x:v>EB-REPORT; coherence/evidence/end_bent_response_review.md, item 08</x:v>
+        <x:v>EB-REPORT; coherence/evidence/end_bent_response_review.md, item 08; coherence/evidence/2026-10-10/source_update.json</x:v>
       </x:c>
       <x:c r="L22" s="28" t="n">
-        <x:v>46304.5</x:v>
+        <x:v>46305</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="67.5" customHeight="1">
@@ -1102,7 +1128,7 @@
         <x:v>MCAD-S1; MCAD-S2; MCAD-DAT1; MCAD-DAT2</x:v>
       </x:c>
       <x:c r="L23" s="28" t="n">
-        <x:v>46304.5</x:v>
+        <x:v>46304</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="67.5" customHeight="1">
@@ -1132,7 +1158,7 @@
         <x:v>PSB-S1; PSB-S2</x:v>
       </x:c>
       <x:c r="L24" s="28" t="n">
-        <x:v>46304.5</x:v>
+        <x:v>46304</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="67.5" customHeight="1">
@@ -1162,10 +1188,10 @@
         <x:v>MCAD-S1; MCAD-S2; GEOMETRY; JOURNAL</x:v>
       </x:c>
       <x:c r="L25" s="28" t="n">
-        <x:v>46304.5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="67.5" customHeight="1">
+        <x:v>46304</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="116" customHeight="1">
       <x:c r="A26" s="24" t="str">
         <x:v>COH-018</x:v>
       </x:c>
@@ -1179,77 +1205,141 @@
         <x:v>Complete notebook comparison</x:v>
       </x:c>
       <x:c r="E26" s="25" t="str">
-        <x:v>The notebook cites the 8 October journal for end-bent inputs. The journal now includes the 9 October pier update. Selected dimensions can be compared automatically; full elevations, offsets and dependencies need review.</x:v>
+        <x:v>Selected cap dimensions match the new saved cases. Geometry notebook still cites the earlier journal; full schedules, elevations, offsets and T006 wind dependencies need review.</x:v>
       </x:c>
       <x:c r="F26" s="25" t="str">
-        <x:v>Reconcile the complete saved geometry inputs and derived schedules with the current journal, documenting agreed conventions.</x:v>
+        <x:v>Reconcile complete saved geometry and derived schedules with accepted T006, documenting conventions.</x:v>
       </x:c>
       <x:c r="G26" s="27"/>
       <x:c r="H26" s="27"/>
       <x:c r="I26" s="28"/>
       <x:c r="J26" s="27"/>
       <x:c r="K26" s="25" t="str">
-        <x:v>GEOMETRY; JOURNAL; ROADWAY</x:v>
+        <x:v>GEOMETRY; JOURNAL; ROADWAY; coherence/evidence/2026-10-10/source_update.json</x:v>
       </x:c>
       <x:c r="L26" s="28" t="n">
-        <x:v>46304.5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="21" customHeight="1">
-      <x:c r="A27" s="18"/>
-      <x:c r="B27" s="27"/>
-      <x:c r="C27" s="19"/>
-      <x:c r="D27" s="19"/>
-      <x:c r="E27" s="19"/>
-      <x:c r="F27" s="19"/>
+        <x:v>46305</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="116" customHeight="1">
+      <x:c r="A27" s="18" t="str">
+        <x:v>COH-019</x:v>
+      </x:c>
+      <x:c r="B27" s="27" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="C27" s="19" t="str">
+        <x:v>Pier</x:v>
+      </x:c>
+      <x:c r="D27" s="19" t="str">
+        <x:v>End-face U-grid pile clearance</x:v>
+      </x:c>
+      <x:c r="E27" s="19" t="str">
+        <x:v>New pier report flags End U grid pile-envelope clearance FAIL. Displayed 2 is a failure flag; the second FAIL is the aggregate actual-cage summary.</x:v>
+      </x:c>
+      <x:c r="F27" s="19" t="str">
+        <x:v>Review and revise the end-face U-grid detail against pile envelopes and fabrication tolerances; regenerate and verify the report.</x:v>
+      </x:c>
       <x:c r="G27" s="27"/>
       <x:c r="H27" s="27"/>
       <x:c r="I27" s="28"/>
       <x:c r="J27" s="27"/>
-      <x:c r="K27" s="19"/>
-      <x:c r="L27" s="28"/>
-    </x:row>
-    <x:row r="28" ht="21" customHeight="1">
-      <x:c r="A28" s="24"/>
-      <x:c r="B28" s="27"/>
-      <x:c r="C28" s="25"/>
-      <x:c r="D28" s="25"/>
-      <x:c r="E28" s="25"/>
-      <x:c r="F28" s="25"/>
+      <x:c r="K27" s="19" t="str">
+        <x:v>PIER-REPORT; PIER-CASE; coherence/evidence/2026-10-10/source_update.json</x:v>
+      </x:c>
+      <x:c r="L27" s="28" t="n">
+        <x:v>46305</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="116" customHeight="1">
+      <x:c r="A28" s="24" t="str">
+        <x:v>COH-020</x:v>
+      </x:c>
+      <x:c r="B28" s="27" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="C28" s="25" t="str">
+        <x:v>End bents</x:v>
+      </x:c>
+      <x:c r="D28" s="25" t="str">
+        <x:v>End-face U-grid pile clearance</x:v>
+      </x:c>
+      <x:c r="E28" s="25" t="str">
+        <x:v>New end-bent report flags End U grid pile-envelope clearance FAIL. Displayed 2 is a failure flag; the second FAIL is the aggregate actual-cage summary.</x:v>
+      </x:c>
+      <x:c r="F28" s="25" t="str">
+        <x:v>Review and revise the end-face U-grid detail and verify it for both ends; regenerate and verify the report.</x:v>
+      </x:c>
       <x:c r="G28" s="27"/>
       <x:c r="H28" s="27"/>
       <x:c r="I28" s="28"/>
       <x:c r="J28" s="27"/>
-      <x:c r="K28" s="25"/>
-      <x:c r="L28" s="28"/>
-    </x:row>
-    <x:row r="29" ht="21" customHeight="1">
-      <x:c r="A29" s="18"/>
-      <x:c r="B29" s="27"/>
-      <x:c r="C29" s="19"/>
-      <x:c r="D29" s="19"/>
-      <x:c r="E29" s="19"/>
-      <x:c r="F29" s="19"/>
+      <x:c r="K28" s="25" t="str">
+        <x:v>EB-REPORT; EB-CASE; coherence/evidence/2026-10-10/source_update.json</x:v>
+      </x:c>
+      <x:c r="L28" s="28" t="n">
+        <x:v>46305</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="116" customHeight="1">
+      <x:c r="A29" s="18" t="str">
+        <x:v>COH-021</x:v>
+      </x:c>
+      <x:c r="B29" s="27" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="C29" s="19" t="str">
+        <x:v>Calculation tool</x:v>
+      </x:c>
+      <x:c r="D29" s="19" t="str">
+        <x:v>Unregistered tool revisions</x:v>
+      </x:c>
+      <x:c r="E29" s="19" t="str">
+        <x:v>The GitHub notebook and local working notebook both differ from the registered CAP-TOOL fingerprint. Their relationship to the supplied report export code is not established.</x:v>
+      </x:c>
+      <x:c r="F29" s="19" t="str">
+        <x:v>Identify the report-generating tool revision, review its changes and consumers, then record an explicit adoption.</x:v>
+      </x:c>
       <x:c r="G29" s="27"/>
       <x:c r="H29" s="27"/>
       <x:c r="I29" s="28"/>
       <x:c r="J29" s="27"/>
-      <x:c r="K29" s="19"/>
-      <x:c r="L29" s="28"/>
-    </x:row>
-    <x:row r="30" ht="21" customHeight="1">
-      <x:c r="A30" s="24"/>
-      <x:c r="B30" s="27"/>
-      <x:c r="C30" s="25"/>
-      <x:c r="D30" s="25"/>
-      <x:c r="E30" s="25"/>
-      <x:c r="F30" s="25"/>
+      <x:c r="K29" s="19" t="str">
+        <x:v>CAP-TOOL; coherence/evidence/2026-10-10/source_update.json</x:v>
+      </x:c>
+      <x:c r="L29" s="28" t="n">
+        <x:v>46305</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="116" customHeight="1">
+      <x:c r="A30" s="24" t="str">
+        <x:v>COH-022</x:v>
+      </x:c>
+      <x:c r="B30" s="27" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="C30" s="25" t="str">
+        <x:v>Journal</x:v>
+      </x:c>
+      <x:c r="D30" s="25" t="str">
+        <x:v>Current cap source references</x:v>
+      </x:c>
+      <x:c r="E30" s="25" t="str">
+        <x:v>T006 journal source notes cite the prior 9 October pier report. Current project reports are the two supplied 10 October snapshots; C005 remains historical by D-003.</x:v>
+      </x:c>
+      <x:c r="F30" s="25" t="str">
+        <x:v>Refresh journal source references through the bounded BPAD workflow when directed; preserve C005 and distinguish selected sources from accepted calculations.</x:v>
+      </x:c>
       <x:c r="G30" s="27"/>
       <x:c r="H30" s="27"/>
       <x:c r="I30" s="28"/>
       <x:c r="J30" s="27"/>
-      <x:c r="K30" s="25"/>
-      <x:c r="L30" s="28"/>
+      <x:c r="K30" s="25" t="str">
+        <x:v>JOURNAL; PIER-REPORT; EB-REPORT; coherence/evidence/2026-10-10/source_update.json</x:v>
+      </x:c>
+      <x:c r="L30" s="28" t="n">
+        <x:v>46305</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="21" customHeight="1">
       <x:c r="A31" s="18"/>
@@ -5572,7 +5662,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf81c45b459b3401e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9de5cc9ec9794190"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Adopt DXF MSE details and centered cheek steel in main bridge model
</commit_message>
<xml_diff>
--- a/project_current/coherence/Coherence_Tracker.xlsx
+++ b/project_current/coherence/Coherence_Tracker.xlsx
@@ -965,8 +965,8 @@
       <c r="L2" s="3"/>
     </row>
     <row r="3" spans="1:12" ht="18.75" customHeight="1">
-      <c r="A3" s="4" t="s">
-        <v>1</v>
+      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="A3" s="4" t="str">
+        <v>Review updated: 14 October 2026. Source selections, recorded responses and closure evidence are preserved here.</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -984,9 +984,9 @@
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="15">
+      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B4" s="15">
         <f>COUNTIFS($A$9:$A$1008,"&lt;&gt;",$B$9:$B$1008,"&lt;&gt;Closed",$B$9:$B$1008,"&lt;&gt;Not applicable")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>3</v>
@@ -1794,19 +1794,39 @@
         <v>46305</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="21" customHeight="1">
-      <c r="A31" s="6"/>
-      <c r="B31" s="12"/>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
-      <c r="F31" s="7"/>
-      <c r="G31" s="12"/>
+    <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="31" spans="1:12" ht="108" customHeight="1">
+      <c r="A31" s="6" t="str">
+        <v>COH-023</v>
+      </c>
+      <c r="B31" s="12" t="str">
+        <v>Open</v>
+      </c>
+      <c r="C31" s="7" t="str">
+        <v>CAD / calculations</v>
+      </c>
+      <c r="D31" s="7" t="str">
+        <v>Reconcile adopted MSE and cheek revision</v>
+      </c>
+      <c r="E31" s="7" t="str">
+        <v>D-026 adopts 235 in end caps, revised walls and single centered #4 cheek mats. Current notebook/report geometry and Figure B8 do not represent these details.</v>
+      </c>
+      <c r="F31" s="7" t="str">
+        <v>Reconcile cap/wall calculations, loads and quantities with adopted CAD. Review anchorage, lug steel and strap interfaces before issuing details.</v>
+      </c>
+      <c r="G31" s="12" t="str">
+        <v>Incorporate all these changes into the main model and add to the project source.</v>
+      </c>
       <c r="H31" s="12"/>
       <c r="I31" s="13"/>
-      <c r="J31" s="12"/>
-      <c r="K31" s="7"/>
-      <c r="L31" s="13"/>
+      <c r="J31" s="12" t="str">
+        <v>CAD adoption verified; calculation reconciliation remains open.</v>
+      </c>
+      <c r="K31" s="7" t="str">
+        <v>D-026; CAD-MODEL; MSE-DETAIL-DXF; EB-CASE; EB2-CASE; BACKWALL-REPORT; GEOMETRY</v>
+      </c>
+      <c r="L31" s="13" t="d">
+        <v>2026-10-14T00:00:00.000Z</v>
+      </c>
     </row>
     <row r="32" spans="1:12" ht="21" customHeight="1">
       <c r="A32" s="9"/>

</xml_diff>

<commit_message>
Update end cap cages across combined cap and cheek envelope
</commit_message>
<xml_diff>
--- a/project_current/coherence/Coherence_Tracker.xlsx
+++ b/project_current/coherence/Coherence_Tracker.xlsx
@@ -986,7 +986,7 @@
       </c>
       <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B4" s="15">
         <f>COUNTIFS($A$9:$A$1008,"&lt;&gt;",$B$9:$B$1008,"&lt;&gt;Closed",$B$9:$B$1008,"&lt;&gt;Not applicable")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>3</v>
@@ -1828,19 +1828,39 @@
         <v>2026-10-14T00:00:00.000Z</v>
       </c>
     </row>
-    <row r="32" spans="1:12" ht="21" customHeight="1">
-      <c r="A32" s="9"/>
-      <c r="B32" s="12"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
-      <c r="G32" s="12"/>
+    <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="32" spans="1:12" ht="108" customHeight="1">
+      <c r="A32" s="9" t="str">
+        <v>COH-024</v>
+      </c>
+      <c r="B32" s="12" t="str">
+        <v>Open</v>
+      </c>
+      <c r="C32" s="10" t="str">
+        <v>CAD / reinforcement</v>
+      </c>
+      <c r="D32" s="10" t="str">
+        <v>Coordinate cap and cheek steel</v>
+      </c>
+      <c r="E32" s="10" t="str">
+        <v>The 251 in cages span the 235 in cap and two 8 in cheeks. New cap steel clashes with unchanged cheek mats: 40 flagged pairs, including four near-tangent numerical results.</v>
+      </c>
+      <c r="F32" s="10" t="str">
+        <v>Review marked views and coordinate cheek bars with cap longitudinal bars and end hoops. Retain all failures until revised geometry and detailing are checked.</v>
+      </c>
+      <c r="G32" s="12" t="str">
+        <v>I ran the cage designs for the out to out distance and expected the cheek wall steel to coincide with the cap steel.</v>
+      </c>
       <c r="H32" s="12"/>
       <c r="I32" s="13"/>
-      <c r="J32" s="12"/>
-      <c r="K32" s="10"/>
-      <c r="L32" s="13"/>
+      <c r="J32" s="12" t="str">
+        <v>62 cap bars per end bent modeled from supplied cases. Concrete and cheek steel unchanged. No clash repair or detailing acceptance yet.</v>
+      </c>
+      <c r="K32" s="10" t="str">
+        <v>D-027; CAD-MODEL; EB-CASE; EB2-CASE; geometry/freecad/evidence/2026-10-14-end-caps/</v>
+      </c>
+      <c r="L32" s="13" t="n">
+        <v>46309</v>
+      </c>
     </row>
     <row r="33" spans="1:12" ht="21" customHeight="1">
       <c r="A33" s="6"/>

</xml_diff>

<commit_message>
Coordinate cheek vertical bars and end cap hoops
</commit_message>
<xml_diff>
--- a/project_current/coherence/Coherence_Tracker.xlsx
+++ b/project_current/coherence/Coherence_Tracker.xlsx
@@ -1828,7 +1828,7 @@
         <v>2026-10-14T00:00:00.000Z</v>
       </c>
     </row>
-    <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="32" spans="1:12" ht="108" customHeight="1">
+    <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="32" spans="1:12" ht="216" customHeight="1">
       <c r="A32" s="9" t="str">
         <v>COH-024</v>
       </c>
@@ -1842,21 +1842,23 @@
         <v>Coordinate cap and cheek steel</v>
       </c>
       <c r="E32" s="10" t="str">
-        <v>The 251 in cages span the 235 in cap and two 8 in cheeks. New cap steel clashes with unchanged cheek mats: 40 flagged pairs, including four near-tangent numerical results.</v>
+        <v>D-028 reduced cap/cheek overlap flags from 40 to 8. Requested vertical-bar and end-hoop changes pass 544 clearance checks. Remaining intersections are the third horizontal cheek bar crossing two cap side bars on each wall.</v>
       </c>
       <c r="F32" s="10" t="str">
-        <v>Review marked views and coordinate cheek bars with cap longitudinal bars and end hoops. Retain all failures until revised geometry and detailing are checked.</v>
+        <v>Coordinate the third horizontal cheek bar with the cap side bars, then rerun physical checks. Keep cover, pile-clearance and other detailing findings open.</v>
       </c>
       <c r="G32" s="12" t="str">
-        <v>I ran the cage designs for the out to out distance and expected the cheek wall steel to coincide with the cap steel.</v>
+        <v>I ran the cage designs for the out to out distance and expected the cheek wall steel to coincide with the cap steel.
+Follow-up: Remove one bar of the close left pair, pull outer verticals inside the long bars, and move the first stirrup inside the cheek mats. They can touch; they cannot clash. Bring them just inside.</v>
       </c>
       <c r="H32" s="12"/>
       <c r="I32" s="13"/>
       <c r="J32" s="12" t="str">
-        <v>62 cap bars per end bent modeled from supplied cases. Concrete and cheek steel unchanged. No clash repair or detailing acceptance yet.</v>
+        <v>D-027: 62 cap bars per end bent modeled from supplied cases. Concrete and cheek steel unchanged. No clash repair or detailing acceptance yet.
+D-028: One vertical removed per cheek, outer verticals moved just inside cap bars, and end hoops moved inward of the mats. 48 cheek bars; 62 cap bars per end. Concrete, other bars and original case files preserved. Eight horizontal-bar intersections remain.</v>
       </c>
       <c r="K32" s="10" t="str">
-        <v>D-027; CAD-MODEL; EB-CASE; EB2-CASE; geometry/freecad/evidence/2026-10-14-end-caps/</v>
+        <v>D-027; CAD-MODEL; EB-CASE; EB2-CASE; geometry/freecad/evidence/2026-10-14-end-caps/; D-028; geometry/freecad/evidence/2026-10-14-cap-cheek-coordination/</v>
       </c>
       <c r="L32" s="13" t="n">
         <v>46309</v>

</xml_diff>

<commit_message>
Lower cheek horizontal row to clear cap bars
</commit_message>
<xml_diff>
--- a/project_current/coherence/Coherence_Tracker.xlsx
+++ b/project_current/coherence/Coherence_Tracker.xlsx
@@ -1828,7 +1828,7 @@
         <v>2026-10-14T00:00:00.000Z</v>
       </c>
     </row>
-    <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="32" spans="1:12" ht="216" customHeight="1">
+    <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="32" spans="1:12" ht="300" customHeight="1">
       <c r="A32" s="9" t="str">
         <v>COH-024</v>
       </c>
@@ -1842,23 +1842,25 @@
         <v>Coordinate cap and cheek steel</v>
       </c>
       <c r="E32" s="10" t="str">
-        <v>D-028 reduced cap/cheek overlap flags from 40 to 8. Requested vertical-bar and end-hoop changes pass 544 clearance checks. Remaining intersections are the third horizontal cheek bar crossing two cap side bars on each wall.</v>
+        <v>D-029 resolves all eight cap/cheek overlaps by lowering MH03 3/8 in on each cheek. Four MH03-MH04 spacings are now 12 3/8 in, exceeding the existing 12 in maximum. These spacing findings remain open by user direction.</v>
       </c>
       <c r="F32" s="10" t="str">
-        <v>Coordinate the third horizontal cheek bar with the cap side bars, then rerun physical checks. Keep cover, pile-clearance and other detailing findings open.</v>
+        <v>Review the four 12 3/8 in horizontal spacings. Other cover, pile-clearance, cap and backwall steel findings remain open.</v>
       </c>
       <c r="G32" s="12" t="str">
         <v>I ran the cage designs for the out to out distance and expected the cheek wall steel to coincide with the cap steel.
-Follow-up: Remove one bar of the close left pair, pull outer verticals inside the long bars, and move the first stirrup inside the cheek mats. They can touch; they cannot clash. Bring them just inside.</v>
+Follow-up: Remove one bar of the close left pair, pull outer verticals inside the long bars, and move the first stirrup inside the cheek mats. They can touch; they cannot clash. Bring them just inside.
+Follow-up: Keep the stirrup at its prior position. Shift only the clashing horizontal row vertically and flag the resulting 12 3/8 in spacing. Keep this revision local.</v>
       </c>
       <c r="H32" s="12"/>
       <c r="I32" s="13"/>
       <c r="J32" s="12" t="str">
         <v>D-027: 62 cap bars per end bent modeled from supplied cases. Concrete and cheek steel unchanged. No clash repair or detailing acceptance yet.
-D-028: One vertical removed per cheek, outer verticals moved just inside cap bars, and end hoops moved inward of the mats. 48 cheek bars; 62 cap bars per end. Concrete, other bars and original case files preserved. Eight horizontal-bar intersections remain.</v>
+D-028: One vertical removed per cheek, outer verticals moved just inside cap bars, and end hoops moved inward of the mats. 48 cheek bars; 62 cap bars per end. Concrete, other bars and original case files preserved. Eight horizontal-bar intersections remain.
+D-029: Lowered only MH03 by 3/8 in at all four cheeks. All eight cap/cheek intersections resolved. Prior stirrup stations and all other bars preserved. Four spacing checks remain FAIL at 12 3/8 in; no threshold relaxed.</v>
       </c>
       <c r="K32" s="10" t="str">
-        <v>D-027; CAD-MODEL; EB-CASE; EB2-CASE; geometry/freecad/evidence/2026-10-14-end-caps/; D-028; geometry/freecad/evidence/2026-10-14-cap-cheek-coordination/</v>
+        <v>D-027; CAD-MODEL; EB-CASE; EB2-CASE; geometry/freecad/evidence/2026-10-14-end-caps/; D-028; geometry/freecad/evidence/2026-10-14-cap-cheek-coordination/; D-029; geometry/freecad/evidence/2026-10-14-horizontal-cheek/</v>
       </c>
       <c r="L32" s="13" t="n">
         <v>46309</v>

</xml_diff>

<commit_message>
Add cheek lug WWR and defer stirrup overlap review
</commit_message>
<xml_diff>
--- a/project_current/coherence/Coherence_Tracker.xlsx
+++ b/project_current/coherence/Coherence_Tracker.xlsx
@@ -986,7 +986,7 @@
       </c>
       <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B4" s="15">
         <f>COUNTIFS($A$9:$A$1008,"&lt;&gt;",$B$9:$B$1008,"&lt;&gt;Closed",$B$9:$B$1008,"&lt;&gt;Not applicable")</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>3</v>
@@ -998,9 +998,9 @@
       <c r="E4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="15">
+      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="F4" s="15">
         <f>COUNTIFS($A$9:$A$1008,"&lt;&gt;",$B$9:$B$1008,"Deferred")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>5</v>
@@ -1866,19 +1866,39 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="33" spans="1:12" ht="21" customHeight="1">
-      <c r="A33" s="6"/>
-      <c r="B33" s="12"/>
-      <c r="C33" s="7"/>
-      <c r="D33" s="7"/>
-      <c r="E33" s="7"/>
-      <c r="F33" s="7"/>
-      <c r="G33" s="12"/>
+    <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="33" spans="1:12" ht="200" customHeight="1">
+      <c r="A33" s="6" t="str">
+        <v>COH-025</v>
+      </c>
+      <c r="B33" s="12" t="str">
+        <v>Deferred</v>
+      </c>
+      <c r="C33" s="7" t="str">
+        <v>CAD / reinforcement</v>
+      </c>
+      <c r="D33" s="7" t="str">
+        <v>End-bent U-bar / hoop overlaps</v>
+      </c>
+      <c r="E33" s="7" t="str">
+        <v>14 overlapping bar pairs remain: seven per end bent at four groups. Turned pile U-bar ends penetrate hoop bottoms. Each pair crosses on both cap sides (14 crossing points per end). Hoop stations: 58.875, 112.875, 166.875 and 192.125 in from the left outer cheek face.</v>
+      </c>
+      <c r="F33" s="7" t="str">
+        <v>Review the U-bar / hoop intersections later and agree revisions. Recheck affected steel, cover, spacing, piles and WWR before closing. Leave current stirrups and U-bars unchanged.</v>
+      </c>
+      <c r="G33" s="12" t="str">
+        <v>Lets leave these clashes for now but flag them for review later in the coherence log</v>
+      </c>
       <c r="H33" s="12"/>
       <c r="I33" s="13"/>
-      <c r="J33" s="12"/>
-      <c r="K33" s="7"/>
-      <c r="L33" s="13"/>
+      <c r="J33" s="12" t="str">
+        <v>Deferred by user on 14 October 2026; unresolved positive-volume overlaps, not accepted as clear. CAD review confirms the same four groups at EB1 and EB2. This deferral concerns these 14 pairs only.</v>
+      </c>
+      <c r="K33" s="7" t="str">
+        <v>CAD-MODEL; EB-CASE; EB2-CASE; geometry/freecad/evidence/2026-10-14-lug-wwr/stirrup-review/; D-030</v>
+      </c>
+      <c r="L33" s="13" t="str">
+        <v>2026-10-14</v>
+      </c>
     </row>
     <row r="34" spans="1:12" ht="21" customHeight="1">
       <c r="A34" s="9"/>

</xml_diff>

<commit_message>
Complete cheek and return connections with slab gap closures and face colors
</commit_message>
<xml_diff>
--- a/project_current/coherence/Coherence_Tracker.xlsx
+++ b/project_current/coherence/Coherence_Tracker.xlsx
@@ -986,7 +986,7 @@
       </c>
       <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B4" s="15">
         <f>COUNTIFS($A$9:$A$1008,"&lt;&gt;",$B$9:$B$1008,"&lt;&gt;Closed",$B$9:$B$1008,"&lt;&gt;Not applicable")</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>3</v>
@@ -1818,8 +1818,8 @@
       </c>
       <c r="H31" s="12"/>
       <c r="I31" s="13"/>
-      <c r="J31" s="12" t="str">
-        <v>CAD adoption verified; calculation reconciliation remains open.</v>
+      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="J31" s="12" t="str">
+        <v>CAD adoption verified; calculation reconciliation remains open. D-033 raises cheek tops to the return bases and deepens transverse return bottoms to the slab. Cheek mats total 52 bars and lug WWR totals 180 wires. Reconcile revised quantities and loads.</v>
       </c>
       <c r="K31" s="7" t="str">
         <v>D-026; CAD-MODEL; MSE-DETAIL-DXF; EB-CASE; EB2-CASE; BACKWALL-REPORT; GEOMETRY</v>
@@ -1900,33 +1900,69 @@
         <v>2026-10-14</v>
       </c>
     </row>
-    <row r="34" spans="1:12" ht="21" customHeight="1">
-      <c r="A34" s="9"/>
-      <c r="B34" s="12"/>
-      <c r="C34" s="10"/>
-      <c r="D34" s="10"/>
-      <c r="E34" s="10"/>
-      <c r="F34" s="10"/>
+    <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="34" spans="1:12" ht="180" customHeight="1">
+      <c r="A34" s="9" t="str">
+        <v>COH-026</v>
+      </c>
+      <c r="B34" s="12" t="str">
+        <v>Open</v>
+      </c>
+      <c r="C34" s="10" t="str">
+        <v>CAD / concrete</v>
+      </c>
+      <c r="D34" s="10" t="str">
+        <v>Coping and MSE wall overlaps</v>
+      </c>
+      <c r="E34" s="10" t="str">
+        <v>Three pre-existing coping/wall intersections remain at A6, A7 and B6. D-033 reduces them to 8,605.016, 1,762.803 and 20,377.450 in3. These are concrete ownership overlaps, separate from steel clashes.</v>
+      </c>
+      <c r="F34" s="10" t="str">
+        <v>Agree concrete ownership and trim the coping/wall interfaces. Recheck concrete quantities and contact geometry.</v>
+      </c>
       <c r="G34" s="12"/>
       <c r="H34" s="12"/>
       <c r="I34" s="13"/>
-      <c r="J34" s="12"/>
-      <c r="K34" s="10"/>
-      <c r="L34" s="13"/>
-    </row>
-    <row r="35" spans="1:12" ht="21" customHeight="1">
-      <c r="A35" s="6"/>
-      <c r="B35" s="12"/>
-      <c r="C35" s="7"/>
-      <c r="D35" s="7"/>
-      <c r="E35" s="7"/>
-      <c r="F35" s="7"/>
+      <c r="J34" s="12" t="str">
+        <v>Native positive-volume intersections confirmed against the prior model. D-033 introduces no new affected concrete or steel intersections. Existing overlaps remain unresolved.</v>
+      </c>
+      <c r="K34" s="10" t="str">
+        <v>D-033; CAD-MODEL; geometry/freecad/evidence/2026-10-15-return-cheeks/concrete-trial.json</v>
+      </c>
+      <c r="L34" s="13" t="d">
+        <v>2026-10-15T00:00:00.000Z</v>
+      </c>
+    </row>
+    <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="35" spans="1:12" ht="180" customHeight="1">
+      <c r="A35" s="6" t="str">
+        <v>COH-027</v>
+      </c>
+      <c r="B35" s="12" t="str">
+        <v>Open</v>
+      </c>
+      <c r="C35" s="7" t="str">
+        <v>CAD / quantities</v>
+      </c>
+      <c r="D35" s="7" t="str">
+        <v>Curved landing volume totals</v>
+      </c>
+      <c r="E35" s="7" t="str">
+        <v>FreeCAD mass properties for both curved landing slabs are not additive. Raw totals decrease after positive material is added. The original slabs already differ from independent triangulated volumes.</v>
+      </c>
+      <c r="F35" s="7" t="str">
+        <v>Reconcile landing quantities using a converged independent volume method before relying on native totals or quantity schedules.</v>
+      </c>
       <c r="G35" s="12"/>
       <c r="H35" s="12"/>
       <c r="I35" s="13"/>
-      <c r="J35" s="12"/>
-      <c r="K35" s="7"/>
-      <c r="L35" s="13"/>
+      <c r="J35" s="12" t="str">
+        <v>D-033 gap checks confirm zero original concrete loss and about 375 / 378 in3 added at A / B. Triangulated volume increases agree. Geometry and contact checks pass; raw quantity totals remain flagged.</v>
+      </c>
+      <c r="K35" s="7" t="str">
+        <v>D-033; CAD-MODEL; geometry/freecad/evidence/2026-10-15-return-cheeks/void-proof.json</v>
+      </c>
+      <c r="L35" s="13" t="d">
+        <v>2026-10-15T00:00:00.000Z</v>
+      </c>
     </row>
     <row r="36" spans="1:12" ht="21" customHeight="1">
       <c r="A36" s="9"/>

</xml_diff>

<commit_message>
Correct curved landing volume reporting with verified integration
</commit_message>
<xml_diff>
--- a/project_current/coherence/Coherence_Tracker.xlsx
+++ b/project_current/coherence/Coherence_Tracker.xlsx
@@ -986,7 +986,7 @@
       </c>
       <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B4" s="15">
         <f>COUNTIFS($A$9:$A$1008,"&lt;&gt;",$B$9:$B$1008,"&lt;&gt;Closed",$B$9:$B$1008,"&lt;&gt;Not applicable")</f>
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>3</v>
@@ -1005,9 +1005,9 @@
       <c r="G4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="15">
+      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="H4" s="15">
         <f>COUNTIFS($A$9:$A$1008,"&lt;&gt;",$B$9:$B$1008,"Closed")+COUNTIFS($A$9:$A$1008,"&lt;&gt;",$B$9:$B$1008,"Not applicable")</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
@@ -1936,8 +1936,8 @@
       <c r="A35" s="6" t="str">
         <v>COH-027</v>
       </c>
-      <c r="B35" s="12" t="str">
-        <v>Open</v>
+      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B35" s="12" t="str">
+        <v>Closed</v>
       </c>
       <c r="C35" s="7" t="str">
         <v>CAD / quantities</v>
@@ -1948,17 +1948,17 @@
       <c r="E35" s="7" t="str">
         <v>FreeCAD mass properties for both curved landing slabs are not additive. Raw totals decrease after positive material is added. The original slabs already differ from independent triangulated volumes.</v>
       </c>
-      <c r="F35" s="7" t="str">
-        <v>Reconcile landing quantities using a converged independent volume method before relying on native totals or quantity schedules.</v>
+      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="F35" s="7" t="str">
+        <v>Completed D-034: use the verified NetVolume property for the two finished landings. The built-in Shape.Volume remains unsuitable for these curved solids.</v>
       </c>
       <c r="G35" s="12"/>
       <c r="H35" s="12"/>
       <c r="I35" s="13"/>
-      <c r="J35" s="12" t="str">
-        <v>D-033 gap checks confirm zero original concrete loss and about 375 / 378 in3 added at A / B. Triangulated volume increases agree. Geometry and contact checks pass; raw quantity totals remain flagged.</v>
-      </c>
-      <c r="K35" s="7" t="str">
-        <v>D-033; CAD-MODEL; geometry/freecad/evidence/2026-10-15-return-cheeks/void-proof.json</v>
+      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="J35" s="12" t="str">
+        <v>D-034: A 111.481112 ft3; B 88.556269 ft3. Adaptive vertical integration passes convergence, independent mesh and added-material checks. Native rebuild/reopen passes. Geometry, steel and colors unchanged.</v>
+      </c>
+      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="K35" s="7" t="str">
+        <v>D-034; CAD-MODEL; geometry/freecad/evidence/2026-10-15-landing-quantities/update-summary.json</v>
       </c>
       <c r="L35" s="13" t="d">
         <v>2026-10-15T00:00:00.000Z</v>

</xml_diff>

<commit_message>
Track FBMP export submittal and pile-head reruns as open items
By user direction, the FBMP XML submittal stays open and the final FBMP
runs are flagged for rerun with updated pile-head elevations.

- COH-013 now covers all three report-matching exports. The pier export
  (c8420fad) was supplied for comparison only and is not submitted.
  End Bent 1 (23bb3afc) and End Bent 2 (56f78267) are missing.
- New COH-028 (Open): rerun the final pier/EB1/EB2 analyses with pile
  heads at the notebook cutoffs 41.764940 / 41.237692 / 41.249692 ft.
  The report-matching pier model is at 41.7717 ft, the pre-D-023 cutoff
  (0.081 in high). D-036 changed no elevations.
- COH-004 is cross-referenced, since its fingerprint statement predates
  the 12 October report.
- Measured evidence record added. The stale FBMP READMEs are corrected.

No export, register row, report or case changed.
</commit_message>
<xml_diff>
--- a/project_current/coherence/Coherence_Tracker.xlsx
+++ b/project_current/coherence/Coherence_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\D2MPDB\project_current\coherence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64C9B1F1-28BD-40DE-8057-E6FF27C16C39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B991146D-38D0-47F9-8E48-98B9C39F2823}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1837" yWindow="1837" windowWidth="18226" windowHeight="11386" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="24496" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Coherence items" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="201">
   <si>
     <t>D2 I-95 project coherence</t>
   </si>
@@ -160,7 +160,10 @@
     <t>Compare the exact current model loading with T006 and document needed reruns and convergence evidence.</t>
   </si>
   <si>
-    <t>PIER-XML; JOURNAL; coherence/evidence/pier_review_2026-10-09.xlsx, item 05; tasks/T006/response-disposition.json, item 05; coherence/evidence/2026-10-10/source_update.json</t>
+    <t>16 Oct: the 12 Oct pier report names export c8420fad..., not the registered PIER-XML (COH-013), and the final runs need the current pile heads (COH-028).</t>
+  </si>
+  <si>
+    <t>PIER-XML; JOURNAL; coherence/evidence/pier_review_2026-10-09.xlsx, item 05; tasks/T006/response-disposition.json, item 05; coherence/evidence/2026-10-10/source_update.json; COH-013; COH-028; coherence/evidence/2026-10-16-fbmp-pile-heads/pile_heads.json</t>
   </si>
   <si>
     <t>COH-005</t>
@@ -313,16 +316,25 @@
     <t>COH-013</t>
   </si>
   <si>
-    <t>Matching raw analysis export</t>
-  </si>
-  <si>
-    <t>New end-bent report requires XML SHA256 8414fbedfbf1270fbd65b2cf940f2dc2050818c282cc6f66db2d20b2f3ff17ee. Available same-named XML matches only the superseded report.</t>
-  </si>
-  <si>
-    <t>Supply the matching new End Bent 1 XML and native run record; do not substitute the older export.</t>
-  </si>
-  <si>
-    <t>EB-REPORT; EB-XML; coherence/evidence/end_bent_provenance.json; coherence/evidence/2026-10-10/source_update.json</t>
+    <t>FBMP</t>
+  </si>
+  <si>
+    <t>Report-matching FBMP exports</t>
+  </si>
+  <si>
+    <t>The selected cap reports name exact raw FBMP exports that are not in project_current. Pier (PIER-REPORT, 12 Oct) requires SHA-256 c8420fad...; the user supplied this file on 16 Oct for comparison only. End Bent 1 (EB-REPORT, 14 Oct) requires 23bb3afc... and End Bent 2 (EB2-REPORT, 14 Oct) requires 56f78267...; neither was supplied. Registered PIER-XML and EB-XML are prior exports matching superseded reports only.</t>
+  </si>
+  <si>
+    <t>Submit the exact XML exports behind the final selected cap reports, with their native run records. After the COH-028 pile-head reruns these are the rerun exports and regenerated reports. Do not substitute older exports.</t>
+  </si>
+  <si>
+    <t>16 Oct: Lets leave the FBMP xml files submittal to the source as an open item.</t>
+  </si>
+  <si>
+    <t>10 Oct: the supplied EB1 export 8414fb... matched the 10 October report. The 12 and 14 October reports then named new exports. 16 Oct: the supplied pier export c8420fad... was compared (pile heads at EL 41.7717 ft, COH-028) and left unsubmitted by user direction. See coherence/evidence/2026-10-16-fbmp-pile-heads/pile_heads.json.</t>
+  </si>
+  <si>
+    <t>EB-REPORT; EB-XML; coherence/evidence/end_bent_provenance.json; coherence/evidence/2026-10-10/source_update.json; PIER-REPORT; PIER-XML; EB2-REPORT; EB2-XML; coherence/evidence/2026-10-12/source_update.json; coherence/evidence/2026-10-16-fbmp-pile-heads/pile_heads.json</t>
   </si>
   <si>
     <t>COH-014</t>
@@ -594,6 +606,27 @@
   </si>
   <si>
     <t>D-034; CAD-MODEL; geometry/freecad/evidence/2026-10-15-landing-quantities/update-summary.json</t>
+  </si>
+  <si>
+    <t>COH-028</t>
+  </si>
+  <si>
+    <t>Rerun final FBMP with current pile heads</t>
+  </si>
+  <si>
+    <t>The 12 Oct D-022/D-023 camber update lowered every notebook pile cutoff by 0.084 in; D-036 changed no elevations. The report-matching pier export (c8420fad..., not submitted) has its pile heads at Z -501.26 in = EL 41.7717 ft, the pre-update cutoff, 0.081 in above the current 41.764940 ft. The 14 Oct end-bent exports cannot be checked (COH-013). Registered prior exports are older models at 41.4175 ft (pier) and 40.3608 ft (EB1).</t>
+  </si>
+  <si>
+    <t>Rerun the final pier, End Bent 1 and End Bent 2 FBMP analyses with pile-head nodes at the notebook cutoffs: pier 41.764940 ft (Z -501.18 in), EB1 41.237692 ft (Z -494.85 in), EB2 41.249692 ft (Z -495.00 in). Confirm pile length, tip and soil inputs, and rerun minimum-tip variants still in use. Regenerate the cap reports and cases, then submit the exports under COH-013.</t>
+  </si>
+  <si>
+    <t>16 Oct: flag the need to rerun the final FBMP runs with updated pile head elevations.</t>
+  </si>
+  <si>
+    <t>Open. Pile heads measured from the export node coordinates and compared with notebook revisions before and after D-023; see coherence/evidence/2026-10-16-fbmp-pile-heads/pile_heads.json.</t>
+  </si>
+  <si>
+    <t>GEOMETRY; D-022; D-023; D-036; PIER-REPORT; PIER-XML; PIER-MINTIP-XML; EB-REPORT; EB-XML; EB-MINTIP-XML; EB2-REPORT; EB2-XML; COH-013; coherence/evidence/2026-10-16-fbmp-pile-heads/pile_heads.json</t>
   </si>
 </sst>
 </file>
@@ -1104,7 +1137,7 @@
       </c>
       <c r="B4" s="15">
         <f>COUNTIFS($A$9:$A$1008,"&lt;&gt;",$B$9:$B$1008,"&lt;&gt;Closed",$B$9:$B$1008,"&lt;&gt;Not applicable")</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>3</v>
@@ -1336,17 +1369,19 @@
       <c r="G12" s="12"/>
       <c r="H12" s="12"/>
       <c r="I12" s="13"/>
-      <c r="J12" s="12"/>
+      <c r="J12" s="12" t="s">
+        <v>46</v>
+      </c>
       <c r="K12" s="10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="L12" s="13">
-        <v>46305</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="116" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B13" s="12" t="s">
         <v>42</v>
@@ -1355,22 +1390,22 @@
         <v>22</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G13" s="12"/>
       <c r="H13" s="12"/>
       <c r="I13" s="13"/>
       <c r="J13" s="12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="L13" s="13">
         <v>46305</v>
@@ -1378,31 +1413,31 @@
     </row>
     <row r="14" spans="1:12" ht="116" customHeight="1">
       <c r="A14" s="9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B14" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G14" s="12"/>
       <c r="H14" s="12"/>
       <c r="I14" s="13"/>
       <c r="J14" s="12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="L14" s="13">
         <v>46305</v>
@@ -1410,7 +1445,7 @@
     </row>
     <row r="15" spans="1:12" ht="116" customHeight="1">
       <c r="A15" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B15" s="12" t="s">
         <v>21</v>
@@ -1419,22 +1454,22 @@
         <v>22</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G15" s="12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H15" s="12"/>
       <c r="I15" s="13"/>
       <c r="J15" s="12"/>
       <c r="K15" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L15" s="13">
         <v>46305</v>
@@ -1442,7 +1477,7 @@
     </row>
     <row r="16" spans="1:12" ht="116" customHeight="1">
       <c r="A16" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B16" s="12" t="s">
         <v>21</v>
@@ -1451,22 +1486,22 @@
         <v>22</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G16" s="12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H16" s="12"/>
       <c r="I16" s="13"/>
       <c r="J16" s="12"/>
       <c r="K16" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="L16" s="13">
         <v>46305</v>
@@ -1474,33 +1509,33 @@
     </row>
     <row r="17" spans="1:12" ht="116" customHeight="1">
       <c r="A17" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B17" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H17" s="12"/>
       <c r="I17" s="13"/>
       <c r="J17" s="12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K17" s="7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="L17" s="13">
         <v>46305</v>
@@ -1508,31 +1543,31 @@
     </row>
     <row r="18" spans="1:12" ht="67.5" customHeight="1">
       <c r="A18" s="9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B18" s="12" t="s">
         <v>4</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G18" s="12" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H18" s="12"/>
       <c r="I18" s="13"/>
       <c r="J18" s="12"/>
       <c r="K18" s="10" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="L18" s="13">
         <v>46304</v>
@@ -1540,31 +1575,31 @@
     </row>
     <row r="19" spans="1:12" ht="116" customHeight="1">
       <c r="A19" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B19" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H19" s="12"/>
       <c r="I19" s="13"/>
       <c r="J19" s="12"/>
       <c r="K19" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="L19" s="13">
         <v>46305</v>
@@ -1572,31 +1607,31 @@
     </row>
     <row r="20" spans="1:12" ht="116" customHeight="1">
       <c r="A20" s="9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B20" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H20" s="12"/>
       <c r="I20" s="13"/>
       <c r="J20" s="12"/>
       <c r="K20" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L20" s="13">
         <v>46305</v>
@@ -1604,61 +1639,65 @@
     </row>
     <row r="21" spans="1:12" ht="116" customHeight="1">
       <c r="A21" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B21" s="12" t="s">
         <v>3</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="G21" s="12"/>
+        <v>101</v>
+      </c>
+      <c r="G21" s="12" t="s">
+        <v>102</v>
+      </c>
       <c r="H21" s="12"/>
       <c r="I21" s="13"/>
-      <c r="J21" s="12"/>
+      <c r="J21" s="12" t="s">
+        <v>103</v>
+      </c>
       <c r="K21" s="7" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="L21" s="13">
-        <v>46305</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="116" customHeight="1">
       <c r="A22" s="9" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B22" s="12" t="s">
         <v>42</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="F22" s="10" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="G22" s="12" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="H22" s="12"/>
       <c r="I22" s="13"/>
       <c r="J22" s="12"/>
       <c r="K22" s="10" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="L22" s="13">
         <v>46305</v>
@@ -1666,31 +1705,31 @@
     </row>
     <row r="23" spans="1:12" ht="67.5" customHeight="1">
       <c r="A23" s="6" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B23" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="H23" s="12"/>
       <c r="I23" s="13"/>
       <c r="J23" s="12"/>
       <c r="K23" s="7" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="L23" s="13">
         <v>46304</v>
@@ -1698,31 +1737,31 @@
     </row>
     <row r="24" spans="1:12" ht="67.5" customHeight="1">
       <c r="A24" s="9" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B24" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="E24" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="G24" s="12" t="s">
         <v>116</v>
-      </c>
-      <c r="F24" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="G24" s="12" t="s">
-        <v>112</v>
       </c>
       <c r="H24" s="12"/>
       <c r="I24" s="13"/>
       <c r="J24" s="12"/>
       <c r="K24" s="10" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="L24" s="13">
         <v>46304</v>
@@ -1730,31 +1769,31 @@
     </row>
     <row r="25" spans="1:12" ht="67.5" customHeight="1">
       <c r="A25" s="6" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B25" s="12" t="s">
         <v>42</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="H25" s="12"/>
       <c r="I25" s="13"/>
       <c r="J25" s="12"/>
       <c r="K25" s="7" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="L25" s="13">
         <v>46304</v>
@@ -1762,29 +1801,29 @@
     </row>
     <row r="26" spans="1:12" ht="116" customHeight="1">
       <c r="A26" s="9" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B26" s="12" t="s">
         <v>42</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="G26" s="12"/>
       <c r="H26" s="12"/>
       <c r="I26" s="13"/>
       <c r="J26" s="12"/>
       <c r="K26" s="10" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="L26" s="13">
         <v>46305</v>
@@ -1792,7 +1831,7 @@
     </row>
     <row r="27" spans="1:12" ht="116" customHeight="1">
       <c r="A27" s="6" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B27" s="12" t="s">
         <v>42</v>
@@ -1801,20 +1840,20 @@
         <v>22</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="G27" s="12"/>
       <c r="H27" s="12"/>
       <c r="I27" s="13"/>
       <c r="J27" s="12"/>
       <c r="K27" s="7" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="L27" s="13">
         <v>46305</v>
@@ -1822,31 +1861,31 @@
     </row>
     <row r="28" spans="1:12" ht="116" customHeight="1">
       <c r="A28" s="9" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B28" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="G28" s="12" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="H28" s="12"/>
       <c r="I28" s="13"/>
       <c r="J28" s="12"/>
       <c r="K28" s="10" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="L28" s="13">
         <v>46305</v>
@@ -1854,29 +1893,29 @@
     </row>
     <row r="29" spans="1:12" ht="116" customHeight="1">
       <c r="A29" s="6" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B29" s="12" t="s">
         <v>42</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="G29" s="12"/>
       <c r="H29" s="12"/>
       <c r="I29" s="13"/>
       <c r="J29" s="12"/>
       <c r="K29" s="7" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="L29" s="13">
         <v>46305</v>
@@ -1884,29 +1923,29 @@
     </row>
     <row r="30" spans="1:12" ht="116" customHeight="1">
       <c r="A30" s="9" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="B30" s="12" t="s">
         <v>42</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="13"/>
       <c r="J30" s="12"/>
       <c r="K30" s="10" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="L30" s="13">
         <v>46305</v>
@@ -1914,33 +1953,33 @@
     </row>
     <row r="31" spans="1:12" ht="108" customHeight="1">
       <c r="A31" s="6" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B31" s="12" t="s">
         <v>42</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="G31" s="12" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="H31" s="12"/>
       <c r="I31" s="13"/>
       <c r="J31" s="12" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="K31" s="7" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="L31" s="13">
         <v>46311</v>
@@ -1948,33 +1987,33 @@
     </row>
     <row r="32" spans="1:12" ht="300" customHeight="1">
       <c r="A32" s="9" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B32" s="12" t="s">
         <v>42</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="F32" s="10" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="G32" s="12" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="H32" s="12"/>
       <c r="I32" s="13"/>
       <c r="J32" s="12" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="K32" s="10" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="L32" s="13">
         <v>46309</v>
@@ -1982,65 +2021,65 @@
     </row>
     <row r="33" spans="1:12" ht="200" customHeight="1">
       <c r="A33" s="6" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="B33" s="12" t="s">
         <v>4</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="G33" s="12" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="H33" s="12"/>
       <c r="I33" s="13"/>
       <c r="J33" s="12" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="K33" s="7" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="L33" s="13" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
     </row>
     <row r="34" spans="1:12" ht="180" customHeight="1">
       <c r="A34" s="9" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B34" s="12" t="s">
         <v>42</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="F34" s="10" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="G34" s="12"/>
       <c r="H34" s="12"/>
       <c r="I34" s="13"/>
       <c r="J34" s="12" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="K34" s="10" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="L34" s="13">
         <v>46310</v>
@@ -2048,49 +2087,69 @@
     </row>
     <row r="35" spans="1:12" ht="180" customHeight="1">
       <c r="A35" s="6" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B35" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="G35" s="12"/>
       <c r="H35" s="12"/>
       <c r="I35" s="13"/>
       <c r="J35" s="12" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="K35" s="7" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="L35" s="13">
         <v>46310</v>
       </c>
     </row>
-    <row r="36" spans="1:12" ht="21" customHeight="1">
-      <c r="A36" s="9"/>
-      <c r="B36" s="12"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="10"/>
-      <c r="G36" s="12"/>
+    <row r="36" spans="1:12" ht="180" customHeight="1">
+      <c r="A36" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="G36" s="12" t="s">
+        <v>198</v>
+      </c>
       <c r="H36" s="12"/>
       <c r="I36" s="13"/>
-      <c r="J36" s="12"/>
-      <c r="K36" s="10"/>
-      <c r="L36" s="13"/>
+      <c r="J36" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="K36" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="L36" s="13">
+        <v>46311</v>
+      </c>
     </row>
     <row r="37" spans="1:12" ht="21" customHeight="1">
       <c r="A37" s="6"/>

</xml_diff>

<commit_message>
Update cheek-wall CAD steel from the selected design report
</commit_message>
<xml_diff>
--- a/project_current/coherence/Coherence_Tracker.xlsx
+++ b/project_current/coherence/Coherence_Tracker.xlsx
@@ -1951,7 +1951,7 @@
         <v>46305</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="108" customHeight="1">
+    <row r="31" spans="1:12" ht="300" customHeight="1">
       <c r="A31" s="6" t="s">
         <v>156</v>
       </c>
@@ -1964,8 +1964,8 @@
       <c r="D31" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="E31" s="7" t="s">
-        <v>159</v>
+      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="E31" s="7" t="str">
+        <v>D-036 geometry and D-037 backwall report now represent the adopted caps and cheeks. D-039 updates CAD cheek mats to the report. Remaining reconciliation covers loads, quantities, anchorage, lug/strap interfaces and the EB1 backwall seat rebuild.</v>
       </c>
       <c r="F31" s="7" t="s">
         <v>160</v>
@@ -1975,17 +1975,18 @@
       </c>
       <c r="H31" s="12"/>
       <c r="I31" s="13"/>
-      <c r="J31" s="12" t="s">
-        <v>162</v>
-      </c>
-      <c r="K31" s="7" t="s">
-        <v>163</v>
+      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="J31" s="12" t="str">
+        <v>CAD adoption verified; calculation reconciliation remains open. D-033 raises cheek tops to the return bases and deepens transverse return bottoms to the slab. Cheek mats total 52 bars and lug WWR totals 180 wires. Reconcile revised quantities and loads. 16 Oct (D-036): the geometry notebook now owns the 235-in caps, backwalls, cheek webs and lugs (cheek tops = D-033 return bases). 105 native station cuts and the cheek/cap volumes match the D-034 CAD solids; the CAD EB1 backwall seat holds 0.117 ft3 more (MSE landing) and is to be rebuilt from the notebook. Cap/wall loads, quantities, anchorage, lug steel and strap interfaces remain open.
+16 Oct (D-039): CAD now has 64 cheek bars, one centered #4 mat at 10 in maximum each way. Physical checks and native reopen pass. Lug WWR remains 180 wires. Other reconciliation remains open.</v>
+      </c>
+      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="K31" s="7" t="str">
+        <v>D-026; CAD-MODEL; MSE-DETAIL-DXF; EB-CASE; EB2-CASE; BACKWALL-REPORT; GEOMETRY; D-036; GEOMETRY-TABLES; D-039; BACKWALL-CASE</v>
       </c>
       <c r="L31" s="13">
         <v>46311</v>
       </c>
     </row>
-    <row r="32" spans="1:12" ht="300" customHeight="1">
+    <row r="32" spans="1:12" ht="400" customHeight="1">
       <c r="A32" s="9" t="s">
         <v>164</v>
       </c>
@@ -1998,25 +1999,28 @@
       <c r="D32" s="10" t="s">
         <v>166</v>
       </c>
-      <c r="E32" s="10" t="s">
-        <v>167</v>
-      </c>
-      <c r="F32" s="10" t="s">
-        <v>168</v>
+      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="E32" s="10" t="str">
+        <v>D-039 replaces the four 12 3/8 in spacing failures with centered #4 mats at 10 in maximum each way. All cheek geometry, cover, spacing, cap-bar and lug-mesh checks pass. Other cap/backwall detailing findings remain open.</v>
+      </c>
+      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="F32" s="10" t="str">
+        <v>Review remaining cap/backwall cover, pile clearance, anchorage and fabrication findings. Cheek spacing and cap/cheek overlap findings are resolved. Keep the separate COH-025 U-bar/hoop deferral.</v>
       </c>
       <c r="G32" s="12" t="s">
         <v>169</v>
       </c>
       <c r="H32" s="12"/>
       <c r="I32" s="13"/>
-      <c r="J32" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="K32" s="10" t="s">
-        <v>171</v>
-      </c>
-      <c r="L32" s="13">
-        <v>46309</v>
+      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="J32" s="12" t="str">
+        <v>D-027: 62 cap bars per end bent modeled from supplied cases. Concrete and cheek steel unchanged. No clash repair or detailing acceptance yet.
+D-028: One vertical removed per cheek, outer verticals moved just inside cap bars, and end hoops moved inward of the mats. 48 cheek bars; 62 cap bars per end. Concrete, other bars and original case files preserved. Eight horizontal-bar intersections remain.
+D-029: Lowered only MH03 by 3/8 in at all four cheeks. All eight cap/cheek intersections resolved. Prior stirrup stations and all other bars preserved. Four spacing checks remain FAIL at 12 3/8 in; no threshold relaxed.
+D-039 (16 Oct): selected report applied to all four cheeks. 64 bars total (5 vertical + 11 horizontal each), 10 in maximum each way. Outer vertical stations retained; inner bars and horizontal phase coordinated with cap steel and WWR. Four spacing failures resolved; no affected overlaps. Cap/backwall/pedestal steel and 180 lug wires preserved.</v>
+      </c>
+      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="K32" s="10" t="str">
+        <v>D-027; CAD-MODEL; EB-CASE; EB2-CASE; geometry/freecad/evidence/2026-10-14-end-caps/; D-028; geometry/freecad/evidence/2026-10-14-cap-cheek-coordination/; D-029; geometry/freecad/evidence/2026-10-14-horizontal-cheek/; D-039; BACKWALL-REPORT; BACKWALL-CASE; geometry/freecad/evidence/2026-10-16-cheek-steel/update-summary.json</v>
+      </c>
+      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L32" s="13" t="d">
+        <v>2026-10-16T00:00:00.000Z</v>
       </c>
     </row>
     <row r="33" spans="1:12" ht="200" customHeight="1">

</xml_diff>

<commit_message>
Tracker: close COH-013 and update COH-004 for the D-073 pier export (D-074)
Coherence_Tracker.xlsx edited in place (project_current/coherence/evidence/
2026-10-21-fbmp/update_tracker.py, rerunnable): COH-013 Closed with the
D-049/D-051/D-073 evidence (every selected cap report and case names a
registered export; analysis-identity checks MATCH), COH-004 kept Open with the
21 October export recorded (loads equal the 19 October export), review date
21 October. Responses, IDs and formulas untouched; recalculated in Excel.
Coherence views, lineage graph and decisions (D-074) refreshed; atlas candidate
prepared, publication pending.
</commit_message>
<xml_diff>
--- a/project_current/coherence/Coherence_Tracker.xlsx
+++ b/project_current/coherence/Coherence_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\D2MPDB\project_current\coherence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B991146D-38D0-47F9-8E48-98B9C39F2823}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DC889B3-6721-4A7A-8A37-38B0BDD06550}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="24496" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
     <t>D2 I-95 project coherence</t>
   </si>
   <si>
-    <t>Review updated: 16 October 2026. Source selections, recorded responses and closure evidence are preserved here.</t>
+    <t>Review updated: 21 October 2026. Source selections, recorded responses and closure evidence are preserved here.</t>
   </si>
   <si>
     <t>Outstanding</t>
@@ -154,16 +154,16 @@
     <t>Complete model load comparison</t>
   </si>
   <si>
-    <t>New Pier_Fixed report/XML fingerprints match and bearing offsets reconcile. Full current wind, below-pad weights, transfer moments, combinations and convergence remain unverified against T006.</t>
+    <t>Pier report/XML fingerprints match (the 10-21 report and case name the registered 21 October export, D-073) and bearing offsets reconcile. The 21 October export carries the same nodal loads as the 19 October one (only the pile material changed to 45 ksi), so the D-062 load review stands. Full current wind, below-pad weights, transfer moments, combinations and convergence remain unverified against T006.</t>
   </si>
   <si>
     <t>Compare the exact current model loading with T006 and document needed reruns and convergence evidence.</t>
   </si>
   <si>
-    <t>16 Oct: the 12 Oct pier report names export c8420fad..., not the registered PIER-XML (COH-013), and the final runs need the current pile heads (COH-028).</t>
-  </si>
-  <si>
-    <t>PIER-XML; JOURNAL; coherence/evidence/pier_review_2026-10-09.xlsx, item 05; tasks/T006/response-disposition.json, item 05; coherence/evidence/2026-10-10/source_update.json; COH-013; COH-028; coherence/evidence/2026-10-16-fbmp-pile-heads/pile_heads.json</t>
+    <t>16 Oct: the 12 Oct pier report names export c8420fad..., not the registered PIER-XML (COH-013), and the final runs need the current pile heads (COH-028). 21 Oct (D-073): the pier export rerun with the 45 ksi pile material is registered and the 10-21 report and case name it (COH-013 closed, D-074); its nodal loads equal the 19 October export (coherence/evidence/2026-10-21-fbmp/source_receipt.json, comparison_with_previous). The full load comparison, native run records and the COH-028 pile-head reruns remain open.</t>
+  </si>
+  <si>
+    <t>PIER-XML; JOURNAL; coherence/evidence/pier_review_2026-10-09.xlsx, item 05; tasks/T006/response-disposition.json, item 05; coherence/evidence/2026-10-10/source_update.json; COH-013; COH-028; coherence/evidence/2026-10-16-fbmp-pile-heads/pile_heads.json; D-062; D-073; coherence/evidence/2026-10-19-fbmp-load-review/fbmp_load_review.md; coherence/evidence/2026-10-21-fbmp/source_receipt.json</t>
   </si>
   <si>
     <t>COH-005</t>
@@ -322,19 +322,19 @@
     <t>Report-matching FBMP exports</t>
   </si>
   <si>
-    <t>The selected cap reports name exact raw FBMP exports that are not in project_current. Pier (PIER-REPORT, 12 Oct) requires SHA-256 c8420fad...; the user supplied this file on 16 Oct for comparison only. End Bent 1 (EB-REPORT, 14 Oct) requires 23bb3afc... and End Bent 2 (EB2-REPORT, 14 Oct) requires 56f78267...; neither was supplied. Registered PIER-XML and EB-XML are prior exports matching superseded reports only.</t>
-  </si>
-  <si>
-    <t>Submit the exact XML exports behind the final selected cap reports, with their native run records. After the COH-028 pile-head reruns these are the rerun exports and regenerated reports. Do not substitute older exports.</t>
+    <t>Resolved: every selected cap report and case names a registered export. End Bent 1 and End Bent 2 (10-19 reports and cases, D-051) name EB-XML and EB2-XML (the 19 October fixed exports, D-049); the pier (10-21 report and case, D-073) names PIER-XML, the 21 October rerun with the 45 ksi pile material (SHA-256 8be45bb889f5...). Historical finding (12 to 16 October): the 12 and 14 October reports named exports that were not in project_current (pier c8420fad..., End Bent 1 23bb3afc..., End Bent 2 56f78267...).</t>
+  </si>
+  <si>
+    <t>None for export identity. Native run records and the pile-head reruns remain under COH-004 and COH-028.</t>
   </si>
   <si>
     <t>16 Oct: Lets leave the FBMP xml files submittal to the source as an open item.</t>
   </si>
   <si>
-    <t>10 Oct: the supplied EB1 export 8414fb... matched the 10 October report. The 12 and 14 October reports then named new exports. 16 Oct: the supplied pier export c8420fad... was compared (pile heads at EL 41.7717 ft, COH-028) and left unsubmitted by user direction. See coherence/evidence/2026-10-16-fbmp-pile-heads/pile_heads.json.</t>
-  </si>
-  <si>
-    <t>EB-REPORT; EB-XML; coherence/evidence/end_bent_provenance.json; coherence/evidence/2026-10-10/source_update.json; PIER-REPORT; PIER-XML; EB2-REPORT; EB2-XML; coherence/evidence/2026-10-12/source_update.json; coherence/evidence/2026-10-16-fbmp-pile-heads/pile_heads.json</t>
+    <t>10 Oct: the supplied EB1 export 8414fb... matched the 10 October report. The 12 and 14 October reports then named new exports. 16 Oct: the supplied pier export c8420fad... was compared (pile heads at EL 41.7717 ft, COH-028) and left unsubmitted by user direction. See coherence/evidence/2026-10-16-fbmp-pile-heads/pile_heads.json. 19 Oct (D-049, D-051): the three fixed exports were registered and the cap notebook rerun on them, so the 10-19 reports and cases name them. 21 Oct (D-073): the rerun pier export is registered and the pier cap and pile cases were rerun from it; machine checks PIER:analysis-identity and EB:analysis-identity read MATCH. Closed by user direction, 21 Oct (D-074). See coherence/evidence/2026-10-21-fbmp/source_receipt.json, 2026-10-21-cap-rerun/source_receipt.json and 2026-10-21-pile-reports/source_receipt.json.</t>
+  </si>
+  <si>
+    <t>EB-REPORT; EB-XML; coherence/evidence/end_bent_provenance.json; coherence/evidence/2026-10-10/source_update.json; PIER-REPORT; PIER-XML; EB2-REPORT; EB2-XML; coherence/evidence/2026-10-12/source_update.json; coherence/evidence/2026-10-16-fbmp-pile-heads/pile_heads.json; D-049; D-051; D-073; D-074; coherence/evidence/2026-10-21-fbmp/source_receipt.json; coherence/evidence/2026-10-21-cap-rerun/source_receipt.json; coherence/machine_checks.json</t>
   </si>
   <si>
     <t>COH-014</t>
@@ -499,7 +499,7 @@
     <t>Reconcile adopted MSE and cheek revision</t>
   </si>
   <si>
-    <t>D-026 adopts 235 in end caps, revised walls and single centered #4 cheek mats. Current notebook/report geometry and Figure B8 do not represent these details.</t>
+    <t>D-036 geometry and D-037 backwall report now represent the adopted caps and cheeks. D-039 updates CAD cheek mats to the report. Remaining reconciliation covers loads, quantities, anchorage, lug/strap interfaces and the EB1 backwall seat rebuild.</t>
   </si>
   <si>
     <t>Reconcile cap/wall calculations, loads and quantities with adopted CAD. Review anchorage, lug steel and strap interfaces before issuing details.</t>
@@ -508,10 +508,11 @@
     <t>Incorporate all these changes into the main model and add to the project source.</t>
   </si>
   <si>
-    <t>CAD adoption verified; calculation reconciliation remains open. D-033 raises cheek tops to the return bases and deepens transverse return bottoms to the slab. Cheek mats total 52 bars and lug WWR totals 180 wires. Reconcile revised quantities and loads. 16 Oct (D-036): the geometry notebook now owns the 235-in caps, backwalls, cheek webs and lugs (cheek tops = D-033 return bases). 105 native station cuts and the cheek/cap volumes match the D-034 CAD solids; the CAD EB1 backwall seat holds 0.117 ft3 more (MSE landing) and is to be rebuilt from the notebook. Cap/wall loads, quantities, anchorage, lug steel and strap interfaces remain open.</t>
-  </si>
-  <si>
-    <t>D-026; CAD-MODEL; MSE-DETAIL-DXF; EB-CASE; EB2-CASE; BACKWALL-REPORT; GEOMETRY; D-036; GEOMETRY-TABLES</t>
+    <t>CAD adoption verified; calculation reconciliation remains open. D-033 raises cheek tops to the return bases and deepens transverse return bottoms to the slab. Cheek mats total 52 bars and lug WWR totals 180 wires. Reconcile revised quantities and loads. 16 Oct (D-036): the geometry notebook now owns the 235-in caps, backwalls, cheek webs and lugs (cheek tops = D-033 return bases). 105 native station cuts and the cheek/cap volumes match the D-034 CAD solids; the CAD EB1 backwall seat holds 0.117 ft3 more (MSE landing) and is to be rebuilt from the notebook. Cap/wall loads, quantities, anchorage, lug steel and strap interfaces remain open.
+16 Oct (D-039): CAD now has 64 cheek bars, one centered #4 mat at 10 in maximum each way. Physical checks and native reopen pass. Lug WWR remains 180 wires. Other reconciliation remains open.</t>
+  </si>
+  <si>
+    <t>D-026; CAD-MODEL; MSE-DETAIL-DXF; EB-CASE; EB2-CASE; BACKWALL-REPORT; GEOMETRY; D-036; GEOMETRY-TABLES; D-039; BACKWALL-CASE</t>
   </si>
   <si>
     <t>COH-024</t>
@@ -523,10 +524,10 @@
     <t>Coordinate cap and cheek steel</t>
   </si>
   <si>
-    <t>D-029 resolves all eight cap/cheek overlaps by lowering MH03 3/8 in on each cheek. Four MH03-MH04 spacings are now 12 3/8 in, exceeding the existing 12 in maximum. These spacing findings remain open by user direction.</t>
-  </si>
-  <si>
-    <t>Review the four 12 3/8 in horizontal spacings. Other cover, pile-clearance, cap and backwall steel findings remain open.</t>
+    <t>D-039 replaces the four 12 3/8 in spacing failures with centered #4 mats at 10 in maximum each way. All cheek geometry, cover, spacing, cap-bar and lug-mesh checks pass. Other cap/backwall detailing findings remain open.</t>
+  </si>
+  <si>
+    <t>Review remaining cap/backwall cover, pile clearance, anchorage and fabrication findings. Cheek spacing and cap/cheek overlap findings are resolved. Keep the separate COH-025 U-bar/hoop deferral.</t>
   </si>
   <si>
     <t>I ran the cage designs for the out to out distance and expected the cheek wall steel to coincide with the cap steel.
@@ -536,10 +537,11 @@
   <si>
     <t>D-027: 62 cap bars per end bent modeled from supplied cases. Concrete and cheek steel unchanged. No clash repair or detailing acceptance yet.
 D-028: One vertical removed per cheek, outer verticals moved just inside cap bars, and end hoops moved inward of the mats. 48 cheek bars; 62 cap bars per end. Concrete, other bars and original case files preserved. Eight horizontal-bar intersections remain.
-D-029: Lowered only MH03 by 3/8 in at all four cheeks. All eight cap/cheek intersections resolved. Prior stirrup stations and all other bars preserved. Four spacing checks remain FAIL at 12 3/8 in; no threshold relaxed.</t>
-  </si>
-  <si>
-    <t>D-027; CAD-MODEL; EB-CASE; EB2-CASE; geometry/freecad/evidence/2026-10-14-end-caps/; D-028; geometry/freecad/evidence/2026-10-14-cap-cheek-coordination/; D-029; geometry/freecad/evidence/2026-10-14-horizontal-cheek/</t>
+D-029: Lowered only MH03 by 3/8 in at all four cheeks. All eight cap/cheek intersections resolved. Prior stirrup stations and all other bars preserved. Four spacing checks remain FAIL at 12 3/8 in; no threshold relaxed.
+D-039 (16 Oct): selected report applied to all four cheeks. 64 bars total (5 vertical + 11 horizontal each), 10 in maximum each way. Outer vertical stations retained; inner bars and horizontal phase coordinated with cap steel and WWR. Four spacing failures resolved; no affected overlaps. Cap/backwall/pedestal steel and 180 lug wires preserved.</t>
+  </si>
+  <si>
+    <t>D-027; CAD-MODEL; EB-CASE; EB2-CASE; geometry/freecad/evidence/2026-10-14-end-caps/; D-028; geometry/freecad/evidence/2026-10-14-cap-cheek-coordination/; D-029; geometry/freecad/evidence/2026-10-14-horizontal-cheek/; D-039; BACKWALL-REPORT; BACKWALL-CASE; geometry/freecad/evidence/2026-10-16-cheek-steel/update-summary.json</t>
   </si>
   <si>
     <t>COH-025</t>
@@ -1137,14 +1139,14 @@
       </c>
       <c r="B4" s="15">
         <f>COUNTIFS($A$9:$A$1008,"&lt;&gt;",$B$9:$B$1008,"&lt;&gt;Closed",$B$9:$B$1008,"&lt;&gt;Not applicable")</f>
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D4" s="15">
         <f>COUNTIFS($A$9:$A$1008,"&lt;&gt;",$B$9:$B$1008,"Awaiting source")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>4</v>
@@ -1158,7 +1160,7 @@
       </c>
       <c r="H4" s="15">
         <f>COUNTIFS($A$9:$A$1008,"&lt;&gt;",$B$9:$B$1008,"Closed")+COUNTIFS($A$9:$A$1008,"&lt;&gt;",$B$9:$B$1008,"Not applicable")</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
@@ -1376,7 +1378,7 @@
         <v>47</v>
       </c>
       <c r="L12" s="13">
-        <v>46311</v>
+        <v>46316</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="116" customHeight="1">
@@ -1642,7 +1644,7 @@
         <v>97</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>98</v>
@@ -1668,7 +1670,7 @@
         <v>104</v>
       </c>
       <c r="L21" s="13">
-        <v>46311</v>
+        <v>46316</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="116" customHeight="1">
@@ -1964,8 +1966,8 @@
       <c r="D31" s="7" t="s">
         <v>158</v>
       </c>
-      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="E31" s="7" t="str">
-        <v>D-036 geometry and D-037 backwall report now represent the adopted caps and cheeks. D-039 updates CAD cheek mats to the report. Remaining reconciliation covers loads, quantities, anchorage, lug/strap interfaces and the EB1 backwall seat rebuild.</v>
+      <c r="E31" s="7" t="s">
+        <v>159</v>
       </c>
       <c r="F31" s="7" t="s">
         <v>160</v>
@@ -1975,18 +1977,17 @@
       </c>
       <c r="H31" s="12"/>
       <c r="I31" s="13"/>
-      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="J31" s="12" t="str">
-        <v>CAD adoption verified; calculation reconciliation remains open. D-033 raises cheek tops to the return bases and deepens transverse return bottoms to the slab. Cheek mats total 52 bars and lug WWR totals 180 wires. Reconcile revised quantities and loads. 16 Oct (D-036): the geometry notebook now owns the 235-in caps, backwalls, cheek webs and lugs (cheek tops = D-033 return bases). 105 native station cuts and the cheek/cap volumes match the D-034 CAD solids; the CAD EB1 backwall seat holds 0.117 ft3 more (MSE landing) and is to be rebuilt from the notebook. Cap/wall loads, quantities, anchorage, lug steel and strap interfaces remain open.
-16 Oct (D-039): CAD now has 64 cheek bars, one centered #4 mat at 10 in maximum each way. Physical checks and native reopen pass. Lug WWR remains 180 wires. Other reconciliation remains open.</v>
-      </c>
-      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="K31" s="7" t="str">
-        <v>D-026; CAD-MODEL; MSE-DETAIL-DXF; EB-CASE; EB2-CASE; BACKWALL-REPORT; GEOMETRY; D-036; GEOMETRY-TABLES; D-039; BACKWALL-CASE</v>
+      <c r="J31" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="K31" s="7" t="s">
+        <v>163</v>
       </c>
       <c r="L31" s="13">
         <v>46311</v>
       </c>
     </row>
-    <row r="32" spans="1:12" ht="400" customHeight="1">
+    <row r="32" spans="1:12" ht="400.05" customHeight="1">
       <c r="A32" s="9" t="s">
         <v>164</v>
       </c>
@@ -1999,28 +2000,25 @@
       <c r="D32" s="10" t="s">
         <v>166</v>
       </c>
-      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="E32" s="10" t="str">
-        <v>D-039 replaces the four 12 3/8 in spacing failures with centered #4 mats at 10 in maximum each way. All cheek geometry, cover, spacing, cap-bar and lug-mesh checks pass. Other cap/backwall detailing findings remain open.</v>
-      </c>
-      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="F32" s="10" t="str">
-        <v>Review remaining cap/backwall cover, pile clearance, anchorage and fabrication findings. Cheek spacing and cap/cheek overlap findings are resolved. Keep the separate COH-025 U-bar/hoop deferral.</v>
+      <c r="E32" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="F32" s="10" t="s">
+        <v>168</v>
       </c>
       <c r="G32" s="12" t="s">
         <v>169</v>
       </c>
       <c r="H32" s="12"/>
       <c r="I32" s="13"/>
-      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="J32" s="12" t="str">
-        <v>D-027: 62 cap bars per end bent modeled from supplied cases. Concrete and cheek steel unchanged. No clash repair or detailing acceptance yet.
-D-028: One vertical removed per cheek, outer verticals moved just inside cap bars, and end hoops moved inward of the mats. 48 cheek bars; 62 cap bars per end. Concrete, other bars and original case files preserved. Eight horizontal-bar intersections remain.
-D-029: Lowered only MH03 by 3/8 in at all four cheeks. All eight cap/cheek intersections resolved. Prior stirrup stations and all other bars preserved. Four spacing checks remain FAIL at 12 3/8 in; no threshold relaxed.
-D-039 (16 Oct): selected report applied to all four cheeks. 64 bars total (5 vertical + 11 horizontal each), 10 in maximum each way. Outer vertical stations retained; inner bars and horizontal phase coordinated with cap steel and WWR. Four spacing failures resolved; no affected overlaps. Cap/backwall/pedestal steel and 180 lug wires preserved.</v>
-      </c>
-      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="K32" s="10" t="str">
-        <v>D-027; CAD-MODEL; EB-CASE; EB2-CASE; geometry/freecad/evidence/2026-10-14-end-caps/; D-028; geometry/freecad/evidence/2026-10-14-cap-cheek-coordination/; D-029; geometry/freecad/evidence/2026-10-14-horizontal-cheek/; D-039; BACKWALL-REPORT; BACKWALL-CASE; geometry/freecad/evidence/2026-10-16-cheek-steel/update-summary.json</v>
-      </c>
-      <c xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L32" s="13" t="d">
-        <v>2026-10-16T00:00:00.000Z</v>
+      <c r="J32" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="K32" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="L32" s="13">
+        <v>46311</v>
       </c>
     </row>
     <row r="33" spans="1:12" ht="200" customHeight="1">

</xml_diff>